<commit_message>
trying to load .nc file
</commit_message>
<xml_diff>
--- a/Output/Data/meta_analysis_data.xlsx
+++ b/Output/Data/meta_analysis_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilylim/Documents/MSc/Course Work/Directed Readings/Meta_Analysis/Output/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilylim/Documents/MSc/Ch2-Meta-analysis/Output/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7708FD96-F156-FB4E-9A6C-9A7185710F28}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8861C88B-D63D-B847-8685-E54242DA9282}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11020" yWindow="460" windowWidth="26780" windowHeight="15940" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
+    <workbookView xWindow="10020" yWindow="2140" windowWidth="26780" windowHeight="15940" activeTab="2" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
   </bookViews>
   <sheets>
     <sheet name="Include" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
adding all rejected papers to csv
</commit_message>
<xml_diff>
--- a/Output/Data/meta_analysis_data.xlsx
+++ b/Output/Data/meta_analysis_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilylim/Documents/MSc/Course Work/Directed Readings/Meta_Analysis/Output/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilylim/Documents/MSc/Ch2-Meta-analysis/Output/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7708FD96-F156-FB4E-9A6C-9A7185710F28}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8861C88B-D63D-B847-8685-E54242DA9282}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11020" yWindow="460" windowWidth="26780" windowHeight="15940" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
+    <workbookView xWindow="10020" yWindow="2140" windowWidth="26780" windowHeight="15940" activeTab="2" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
   </bookViews>
   <sheets>
     <sheet name="Include" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
change the last Pfister experiment to have the same paper_num as the other two experiments in the same paper
</commit_message>
<xml_diff>
--- a/Output/Data/meta_analysis_data.xlsx
+++ b/Output/Data/meta_analysis_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilylim/Documents/MSc/Ch2-Meta-analysis/Output/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8861C88B-D63D-B847-8685-E54242DA9282}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B47F9B81-BDD6-5F41-A566-200BDC1B9B52}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10020" yWindow="2140" windowWidth="26780" windowHeight="15940" activeTab="2" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
+    <workbookView xWindow="6820" yWindow="2140" windowWidth="26780" windowHeight="15940" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
   </bookViews>
   <sheets>
     <sheet name="Include" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7283" uniqueCount="1200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7283" uniqueCount="1199">
   <si>
     <t>paper_num</t>
   </si>
@@ -3072,9 +3072,6 @@
   </si>
   <si>
     <t>Halymeniaceae</t>
-  </si>
-  <si>
-    <t>spring-summer</t>
   </si>
   <si>
     <t>August 9th</t>
@@ -4468,7 +4465,7 @@
         <v>586</v>
       </c>
       <c r="AP1" s="1" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="AQ1" s="1" t="s">
         <v>320</v>
@@ -5087,16 +5084,16 @@
         <v>313</v>
       </c>
       <c r="AC6" s="11" t="s">
+        <v>936</v>
+      </c>
+      <c r="AD6" s="11" t="s">
         <v>937</v>
       </c>
-      <c r="AD6" s="11" t="s">
+      <c r="AE6" s="11" t="s">
+        <v>959</v>
+      </c>
+      <c r="AF6" s="11" t="s">
         <v>938</v>
-      </c>
-      <c r="AE6" s="11" t="s">
-        <v>960</v>
-      </c>
-      <c r="AF6" s="11" t="s">
-        <v>939</v>
       </c>
       <c r="AG6" s="11" t="s">
         <v>923</v>
@@ -5230,16 +5227,16 @@
         <v>313</v>
       </c>
       <c r="AC7" s="11" t="s">
+        <v>936</v>
+      </c>
+      <c r="AD7" s="11" t="s">
         <v>937</v>
       </c>
-      <c r="AD7" s="11" t="s">
+      <c r="AE7" s="11" t="s">
+        <v>959</v>
+      </c>
+      <c r="AF7" s="11" t="s">
         <v>938</v>
-      </c>
-      <c r="AE7" s="11" t="s">
-        <v>960</v>
-      </c>
-      <c r="AF7" s="11" t="s">
-        <v>939</v>
       </c>
       <c r="AG7" s="11" t="s">
         <v>923</v>
@@ -5388,7 +5385,7 @@
         <v>898</v>
       </c>
       <c r="AH8" s="1" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="AI8" s="1" t="s">
         <v>362</v>
@@ -5397,7 +5394,7 @@
         <v>800</v>
       </c>
       <c r="AK8" s="1" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="AL8" s="11" t="s">
         <v>315</v>
@@ -5531,7 +5528,7 @@
         <v>898</v>
       </c>
       <c r="AH9" s="1" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="AI9" s="1" t="s">
         <v>362</v>
@@ -5659,22 +5656,22 @@
         <v>313</v>
       </c>
       <c r="AC10" s="11" t="s">
+        <v>936</v>
+      </c>
+      <c r="AD10" s="11" t="s">
         <v>937</v>
       </c>
-      <c r="AD10" s="11" t="s">
+      <c r="AE10" s="11" t="s">
+        <v>959</v>
+      </c>
+      <c r="AF10" s="11" t="s">
         <v>938</v>
-      </c>
-      <c r="AE10" s="11" t="s">
-        <v>960</v>
-      </c>
-      <c r="AF10" s="11" t="s">
-        <v>939</v>
       </c>
       <c r="AG10" s="11" t="s">
         <v>923</v>
       </c>
       <c r="AH10" s="11" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="AI10" s="11" t="s">
         <v>362</v>
@@ -5713,7 +5710,7 @@
         <v>9</v>
       </c>
       <c r="AU10" s="1" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
     </row>
     <row r="11" spans="1:47">
@@ -5802,22 +5799,22 @@
         <v>313</v>
       </c>
       <c r="AC11" s="11" t="s">
+        <v>936</v>
+      </c>
+      <c r="AD11" s="11" t="s">
         <v>937</v>
       </c>
-      <c r="AD11" s="11" t="s">
+      <c r="AE11" s="11" t="s">
+        <v>959</v>
+      </c>
+      <c r="AF11" s="11" t="s">
         <v>938</v>
-      </c>
-      <c r="AE11" s="11" t="s">
-        <v>960</v>
-      </c>
-      <c r="AF11" s="11" t="s">
-        <v>939</v>
       </c>
       <c r="AG11" s="11" t="s">
         <v>923</v>
       </c>
       <c r="AH11" s="11" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="AI11" s="11" t="s">
         <v>362</v>
@@ -5856,7 +5853,7 @@
         <v>9</v>
       </c>
       <c r="AU11" s="1" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
     </row>
     <row r="12" spans="1:47">
@@ -5960,7 +5957,7 @@
         <v>898</v>
       </c>
       <c r="AH12" s="11" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="AI12" s="11" t="s">
         <v>362</v>
@@ -5969,7 +5966,7 @@
         <v>800</v>
       </c>
       <c r="AK12" s="11" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="AL12" s="11" t="s">
         <v>315</v>
@@ -5999,7 +5996,7 @@
         <v>9</v>
       </c>
       <c r="AU12" s="1" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
     </row>
     <row r="13" spans="1:47">
@@ -6103,7 +6100,7 @@
         <v>898</v>
       </c>
       <c r="AH13" s="11" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="AI13" s="11" t="s">
         <v>362</v>
@@ -6142,7 +6139,7 @@
         <v>9</v>
       </c>
       <c r="AU13" s="1" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
     </row>
     <row r="14" spans="1:47">
@@ -6328,7 +6325,7 @@
         <v>424</v>
       </c>
       <c r="Q15" s="1" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="R15" s="1" t="s">
         <v>315</v>
@@ -6340,7 +6337,7 @@
         <v>315</v>
       </c>
       <c r="U15" s="1" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="V15" s="1" t="s">
         <v>295</v>
@@ -6355,16 +6352,16 @@
         <v>581</v>
       </c>
       <c r="Z15" s="1" t="s">
+        <v>974</v>
+      </c>
+      <c r="AA15" s="1" t="s">
         <v>975</v>
-      </c>
-      <c r="AA15" s="1" t="s">
-        <v>976</v>
       </c>
       <c r="AB15" s="1" t="s">
         <v>295</v>
       </c>
       <c r="AC15" s="1" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="AD15" s="1" t="s">
         <v>662</v>
@@ -6373,10 +6370,10 @@
         <v>601</v>
       </c>
       <c r="AF15" s="1" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="AG15" s="1" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="AH15" s="1" t="s">
         <v>615</v>
@@ -6418,7 +6415,7 @@
         <v>12</v>
       </c>
       <c r="AU15" s="1" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
     </row>
     <row r="16" spans="1:47">
@@ -6471,7 +6468,7 @@
         <v>424</v>
       </c>
       <c r="Q16" s="1" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="R16" s="1" t="s">
         <v>315</v>
@@ -6483,7 +6480,7 @@
         <v>315</v>
       </c>
       <c r="U16" s="1" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="V16" s="1" t="s">
         <v>295</v>
@@ -6498,16 +6495,16 @@
         <v>581</v>
       </c>
       <c r="Z16" s="1" t="s">
+        <v>974</v>
+      </c>
+      <c r="AA16" s="1" t="s">
         <v>975</v>
-      </c>
-      <c r="AA16" s="1" t="s">
-        <v>976</v>
       </c>
       <c r="AB16" s="1" t="s">
         <v>295</v>
       </c>
       <c r="AC16" s="1" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="AD16" s="1" t="s">
         <v>662</v>
@@ -6516,10 +6513,10 @@
         <v>601</v>
       </c>
       <c r="AF16" s="1" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="AG16" s="1" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="AH16" s="1" t="s">
         <v>640</v>
@@ -6561,7 +6558,7 @@
         <v>12</v>
       </c>
       <c r="AU16" s="1" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
     </row>
     <row r="17" spans="1:47">
@@ -6704,7 +6701,7 @@
         <v>3</v>
       </c>
       <c r="AU17" s="1" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="18" spans="1:47">
@@ -6847,7 +6844,7 @@
         <v>3</v>
       </c>
       <c r="AU18" s="1" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="19" spans="1:47">
@@ -7928,7 +7925,7 @@
         <v>723</v>
       </c>
       <c r="AG26" s="1" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="AH26" s="1" t="s">
         <v>593</v>
@@ -7970,7 +7967,7 @@
         <v>5</v>
       </c>
       <c r="AU26" s="1" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="27" spans="1:47">
@@ -8068,7 +8065,7 @@
         <v>723</v>
       </c>
       <c r="AG27" s="1" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="AH27" s="1" t="s">
         <v>593</v>
@@ -8110,7 +8107,7 @@
         <v>8</v>
       </c>
       <c r="AU27" s="1" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="28" spans="1:47">
@@ -8208,7 +8205,7 @@
         <v>723</v>
       </c>
       <c r="AG28" s="1" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="AH28" s="1" t="s">
         <v>593</v>
@@ -8250,7 +8247,7 @@
         <v>3</v>
       </c>
       <c r="AU28" s="1" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="29" spans="1:47">
@@ -8348,7 +8345,7 @@
         <v>723</v>
       </c>
       <c r="AG29" s="1" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="AH29" s="1" t="s">
         <v>593</v>
@@ -8390,7 +8387,7 @@
         <v>4</v>
       </c>
       <c r="AU29" s="1" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="30" spans="1:47">
@@ -8488,7 +8485,7 @@
         <v>723</v>
       </c>
       <c r="AG30" s="1" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="AH30" s="1" t="s">
         <v>593</v>
@@ -8530,7 +8527,7 @@
         <v>4</v>
       </c>
       <c r="AU30" s="1" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="31" spans="1:47">
@@ -8583,7 +8580,7 @@
         <v>294</v>
       </c>
       <c r="Q31" s="1" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
       <c r="R31" s="1" t="s">
         <v>315</v>
@@ -8601,7 +8598,7 @@
         <v>295</v>
       </c>
       <c r="W31" s="1" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
       <c r="X31" s="1" t="s">
         <v>662</v>
@@ -8610,16 +8607,16 @@
         <v>663</v>
       </c>
       <c r="Z31" s="1" t="s">
+        <v>1102</v>
+      </c>
+      <c r="AA31" s="1" t="s">
         <v>1103</v>
-      </c>
-      <c r="AA31" s="1" t="s">
-        <v>1104</v>
       </c>
       <c r="AB31" s="1" t="s">
         <v>295</v>
       </c>
       <c r="AC31" s="1" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
       <c r="AD31" s="1" t="s">
         <v>618</v>
@@ -8628,10 +8625,10 @@
         <v>621</v>
       </c>
       <c r="AF31" s="1" t="s">
+        <v>1099</v>
+      </c>
+      <c r="AG31" s="1" t="s">
         <v>1100</v>
-      </c>
-      <c r="AG31" s="1" t="s">
-        <v>1101</v>
       </c>
       <c r="AH31" s="1" t="s">
         <v>715</v>
@@ -8673,7 +8670,7 @@
         <v>10</v>
       </c>
       <c r="AU31" s="1" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="32" spans="1:47">
@@ -9167,7 +9164,7 @@
         <v>315</v>
       </c>
       <c r="U35" s="11" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="V35" s="1" t="s">
         <v>345</v>
@@ -9242,7 +9239,7 @@
         <v>15</v>
       </c>
       <c r="AU35" s="1" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="36" spans="1:47">
@@ -9307,7 +9304,7 @@
         <v>315</v>
       </c>
       <c r="U36" s="11" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="V36" s="1" t="s">
         <v>345</v>
@@ -9334,10 +9331,10 @@
         <v>315</v>
       </c>
       <c r="AD36" s="1" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="AE36" s="1" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="AF36" s="1" t="s">
         <v>315</v>
@@ -9382,7 +9379,7 @@
         <v>15</v>
       </c>
       <c r="AU36" s="1" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="37" spans="1:47">
@@ -9447,7 +9444,7 @@
         <v>315</v>
       </c>
       <c r="U37" s="11" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="V37" s="1" t="s">
         <v>345</v>
@@ -9474,10 +9471,10 @@
         <v>315</v>
       </c>
       <c r="AD37" s="1" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="AE37" s="1" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="AF37" s="1" t="s">
         <v>315</v>
@@ -9522,7 +9519,7 @@
         <v>15</v>
       </c>
       <c r="AU37" s="1" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="38" spans="1:47">
@@ -9587,7 +9584,7 @@
         <v>315</v>
       </c>
       <c r="U38" s="11" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="V38" s="1" t="s">
         <v>345</v>
@@ -9614,10 +9611,10 @@
         <v>315</v>
       </c>
       <c r="AD38" s="1" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="AE38" s="1" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="AF38" s="1" t="s">
         <v>315</v>
@@ -9662,7 +9659,7 @@
         <v>15</v>
       </c>
       <c r="AU38" s="1" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="39" spans="1:47">
@@ -9727,7 +9724,7 @@
         <v>315</v>
       </c>
       <c r="U39" s="11" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="V39" s="1" t="s">
         <v>345</v>
@@ -9802,7 +9799,7 @@
         <v>15</v>
       </c>
       <c r="AU39" s="1" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="40" spans="1:47">
@@ -9867,7 +9864,7 @@
         <v>315</v>
       </c>
       <c r="U40" s="11" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="V40" s="1" t="s">
         <v>345</v>
@@ -9942,7 +9939,7 @@
         <v>15</v>
       </c>
       <c r="AU40" s="1" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="41" spans="1:47">
@@ -10007,7 +10004,7 @@
         <v>315</v>
       </c>
       <c r="U41" s="11" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="V41" s="1" t="s">
         <v>345</v>
@@ -10082,7 +10079,7 @@
         <v>15</v>
       </c>
       <c r="AU41" s="1" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="42" spans="1:47">
@@ -10195,7 +10192,7 @@
         <v>722</v>
       </c>
       <c r="AK42" s="1" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="AL42" s="1" t="s">
         <v>315</v>
@@ -10225,7 +10222,7 @@
         <v>50</v>
       </c>
       <c r="AU42" s="1" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="43" spans="1:47">
@@ -10338,7 +10335,7 @@
         <v>722</v>
       </c>
       <c r="AK43" s="1" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="AL43" s="1" t="s">
         <v>315</v>
@@ -10368,7 +10365,7 @@
         <v>60</v>
       </c>
       <c r="AU43" s="1" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="44" spans="1:47">
@@ -10481,7 +10478,7 @@
         <v>722</v>
       </c>
       <c r="AK44" s="1" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="AL44" s="1" t="s">
         <v>315</v>
@@ -10511,7 +10508,7 @@
         <v>60</v>
       </c>
       <c r="AU44" s="1" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="45" spans="1:47">
@@ -10624,7 +10621,7 @@
         <v>722</v>
       </c>
       <c r="AK45" s="1" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="AL45" s="1" t="s">
         <v>315</v>
@@ -10654,7 +10651,7 @@
         <v>60</v>
       </c>
       <c r="AU45" s="1" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="46" spans="1:47">
@@ -10767,7 +10764,7 @@
         <v>722</v>
       </c>
       <c r="AK46" s="1" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="AL46" s="1" t="s">
         <v>315</v>
@@ -10797,7 +10794,7 @@
         <v>60</v>
       </c>
       <c r="AU46" s="1" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="47" spans="1:47">
@@ -10910,7 +10907,7 @@
         <v>722</v>
       </c>
       <c r="AK47" s="1" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="AL47" s="1" t="s">
         <v>315</v>
@@ -10940,7 +10937,7 @@
         <v>50</v>
       </c>
       <c r="AU47" s="1" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="48" spans="1:47">
@@ -11053,7 +11050,7 @@
         <v>722</v>
       </c>
       <c r="AK48" s="1" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="AL48" s="1" t="s">
         <v>315</v>
@@ -11083,7 +11080,7 @@
         <v>60</v>
       </c>
       <c r="AU48" s="1" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="49" spans="1:47">
@@ -11196,7 +11193,7 @@
         <v>722</v>
       </c>
       <c r="AK49" s="1" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="AL49" s="1" t="s">
         <v>315</v>
@@ -11226,7 +11223,7 @@
         <v>60</v>
       </c>
       <c r="AU49" s="1" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
     </row>
     <row r="50" spans="1:47">
@@ -11339,7 +11336,7 @@
         <v>722</v>
       </c>
       <c r="AK50" s="1" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="AL50" s="1" t="s">
         <v>315</v>
@@ -11369,7 +11366,7 @@
         <v>60</v>
       </c>
       <c r="AU50" s="1" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="51" spans="1:47">
@@ -11482,7 +11479,7 @@
         <v>722</v>
       </c>
       <c r="AK51" s="1" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="AL51" s="1" t="s">
         <v>315</v>
@@ -11512,7 +11509,7 @@
         <v>60</v>
       </c>
       <c r="AU51" s="1" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="52" spans="1:47">
@@ -17316,10 +17313,10 @@
         <v>315</v>
       </c>
       <c r="AD92" s="1" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="AE92" s="1" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="AF92" s="1" t="s">
         <v>315</v>
@@ -17337,7 +17334,7 @@
         <v>800</v>
       </c>
       <c r="AK92" s="1" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="AL92" s="1" t="s">
         <v>671</v>
@@ -17367,7 +17364,7 @@
         <v>4</v>
       </c>
       <c r="AU92" s="1" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="93" spans="1:47">
@@ -17510,7 +17507,7 @@
         <v>3</v>
       </c>
       <c r="AU93" s="1" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
     </row>
     <row r="94" spans="1:47">
@@ -18043,7 +18040,7 @@
         <v>600</v>
       </c>
       <c r="AH97" s="1" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="AI97" s="1" t="s">
         <v>362</v>
@@ -18901,7 +18898,7 @@
         <v>362</v>
       </c>
       <c r="AJ103" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK103" s="1" t="s">
         <v>832</v>
@@ -18934,7 +18931,7 @@
         <v>10</v>
       </c>
       <c r="AU103" s="1" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="104" spans="1:47">
@@ -19038,7 +19035,7 @@
         <v>362</v>
       </c>
       <c r="AJ104" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK104" s="1" t="s">
         <v>832</v>
@@ -19071,7 +19068,7 @@
         <v>10</v>
       </c>
       <c r="AU104" s="1" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="105" spans="1:47">
@@ -19175,7 +19172,7 @@
         <v>362</v>
       </c>
       <c r="AJ105" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK105" s="1" t="s">
         <v>832</v>
@@ -19208,7 +19205,7 @@
         <v>10</v>
       </c>
       <c r="AU105" s="1" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="106" spans="1:47">
@@ -19312,7 +19309,7 @@
         <v>362</v>
       </c>
       <c r="AJ106" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK106" s="1" t="s">
         <v>832</v>
@@ -19345,7 +19342,7 @@
         <v>10</v>
       </c>
       <c r="AU106" s="1" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="107" spans="1:47">
@@ -19449,7 +19446,7 @@
         <v>362</v>
       </c>
       <c r="AJ107" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK107" s="1" t="s">
         <v>832</v>
@@ -19482,7 +19479,7 @@
         <v>10</v>
       </c>
       <c r="AU107" s="1" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="108" spans="1:47">
@@ -19586,7 +19583,7 @@
         <v>362</v>
       </c>
       <c r="AJ108" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK108" s="1" t="s">
         <v>832</v>
@@ -19619,7 +19616,7 @@
         <v>10</v>
       </c>
       <c r="AU108" s="1" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="109" spans="1:47">
@@ -19723,7 +19720,7 @@
         <v>362</v>
       </c>
       <c r="AJ109" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK109" s="1" t="s">
         <v>832</v>
@@ -19756,7 +19753,7 @@
         <v>10</v>
       </c>
       <c r="AU109" s="1" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="110" spans="1:47">
@@ -19860,7 +19857,7 @@
         <v>362</v>
       </c>
       <c r="AJ110" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK110" s="1" t="s">
         <v>832</v>
@@ -19893,7 +19890,7 @@
         <v>9</v>
       </c>
       <c r="AU110" s="1" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="111" spans="1:47">
@@ -19997,7 +19994,7 @@
         <v>362</v>
       </c>
       <c r="AJ111" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK111" s="1" t="s">
         <v>832</v>
@@ -20030,7 +20027,7 @@
         <v>9</v>
       </c>
       <c r="AU111" s="1" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="112" spans="1:47">
@@ -20134,7 +20131,7 @@
         <v>362</v>
       </c>
       <c r="AJ112" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK112" s="1" t="s">
         <v>832</v>
@@ -20167,7 +20164,7 @@
         <v>9</v>
       </c>
       <c r="AU112" s="1" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="113" spans="1:47">
@@ -20271,7 +20268,7 @@
         <v>362</v>
       </c>
       <c r="AJ113" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK113" s="1" t="s">
         <v>832</v>
@@ -20304,7 +20301,7 @@
         <v>9</v>
       </c>
       <c r="AU113" s="1" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="114" spans="1:47">
@@ -20408,7 +20405,7 @@
         <v>362</v>
       </c>
       <c r="AJ114" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK114" s="1" t="s">
         <v>832</v>
@@ -20441,7 +20438,7 @@
         <v>9</v>
       </c>
       <c r="AU114" s="1" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="115" spans="1:47" customFormat="1">
@@ -20551,7 +20548,7 @@
         <v>362</v>
       </c>
       <c r="AJ115" s="1" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="AK115" s="1" t="s">
         <v>584</v>
@@ -20584,7 +20581,7 @@
         <v>5</v>
       </c>
       <c r="AU115" s="1" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="116" spans="1:47" customFormat="1">
@@ -20694,7 +20691,7 @@
         <v>362</v>
       </c>
       <c r="AJ116" s="1" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="AK116" s="1" t="s">
         <v>584</v>
@@ -20727,7 +20724,7 @@
         <v>5</v>
       </c>
       <c r="AU116" s="1" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="117" spans="1:47" customFormat="1">
@@ -20837,10 +20834,10 @@
         <v>362</v>
       </c>
       <c r="AJ117" s="1" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="AK117" s="1" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
       <c r="AL117" s="1" t="s">
         <v>315</v>
@@ -20870,7 +20867,7 @@
         <v>5</v>
       </c>
       <c r="AU117" s="1" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="118" spans="1:47" customFormat="1">
@@ -20980,10 +20977,10 @@
         <v>362</v>
       </c>
       <c r="AJ118" s="1" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="AK118" s="1" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
       <c r="AL118" s="1" t="s">
         <v>315</v>
@@ -21013,7 +21010,7 @@
         <v>5</v>
       </c>
       <c r="AU118" s="1" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="119" spans="1:47" customFormat="1">
@@ -21117,16 +21114,16 @@
         <v>813</v>
       </c>
       <c r="AH119" s="1" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="AI119" s="1" t="s">
         <v>362</v>
       </c>
       <c r="AJ119" s="1" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="AK119" s="1" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
       <c r="AL119" s="1" t="s">
         <v>315</v>
@@ -21156,7 +21153,7 @@
         <v>5</v>
       </c>
       <c r="AU119" s="1" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="120" spans="1:47" customFormat="1">
@@ -21260,16 +21257,16 @@
         <v>813</v>
       </c>
       <c r="AH120" s="1" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="AI120" s="1" t="s">
         <v>362</v>
       </c>
       <c r="AJ120" s="1" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="AK120" s="1" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
       <c r="AL120" s="1" t="s">
         <v>315</v>
@@ -21299,7 +21296,7 @@
         <v>5</v>
       </c>
       <c r="AU120" s="1" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="121" spans="1:47">
@@ -24150,7 +24147,7 @@
         <v>295</v>
       </c>
       <c r="W141" s="1" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="X141" s="1" t="s">
         <v>885</v>
@@ -24171,10 +24168,10 @@
         <v>315</v>
       </c>
       <c r="AD141" s="1" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="AE141" s="1" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="AF141" s="1" t="s">
         <v>315</v>
@@ -24222,7 +24219,7 @@
         <v>4</v>
       </c>
       <c r="AU141" s="7" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
     </row>
     <row r="142" spans="1:47">
@@ -24308,28 +24305,28 @@
         <v>295</v>
       </c>
       <c r="AC142" s="1" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
       <c r="AD142" s="1" t="s">
         <v>347</v>
       </c>
       <c r="AE142" s="1" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="AF142" s="1" t="s">
+        <v>1072</v>
+      </c>
+      <c r="AG142" s="1" t="s">
         <v>1073</v>
       </c>
-      <c r="AG142" s="1" t="s">
-        <v>1074</v>
-      </c>
       <c r="AH142" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AI142" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AJ142" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK142" s="1" t="s">
         <v>318</v>
@@ -24362,7 +24359,7 @@
         <v>3</v>
       </c>
       <c r="AU142" s="1" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="143" spans="1:47">
@@ -24448,28 +24445,28 @@
         <v>295</v>
       </c>
       <c r="AC143" s="1" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="AD143" s="1" t="s">
         <v>347</v>
       </c>
       <c r="AE143" s="1" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="AF143" s="1" t="s">
+        <v>1081</v>
+      </c>
+      <c r="AG143" s="1" t="s">
+        <v>1075</v>
+      </c>
+      <c r="AH143" s="1" t="s">
         <v>1082</v>
       </c>
-      <c r="AG143" s="1" t="s">
-        <v>1076</v>
-      </c>
-      <c r="AH143" s="1" t="s">
-        <v>1083</v>
-      </c>
       <c r="AI143" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AJ143" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK143" s="1" t="s">
         <v>318</v>
@@ -24502,7 +24499,7 @@
         <v>3</v>
       </c>
       <c r="AU143" s="1" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="144" spans="1:47">
@@ -24588,7 +24585,7 @@
         <v>295</v>
       </c>
       <c r="AC144" s="1" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="AD144" s="1" t="s">
         <v>347</v>
@@ -24597,19 +24594,19 @@
         <v>348</v>
       </c>
       <c r="AF144" s="1" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="AG144" s="1" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="AH144" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AI144" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AJ144" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK144" s="1" t="s">
         <v>318</v>
@@ -24642,7 +24639,7 @@
         <v>3</v>
       </c>
       <c r="AU144" s="1" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="145" spans="1:47">
@@ -24740,16 +24737,16 @@
         <v>842</v>
       </c>
       <c r="AG145" s="1" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="AH145" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AI145" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AJ145" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK145" s="1" t="s">
         <v>318</v>
@@ -24782,7 +24779,7 @@
         <v>3</v>
       </c>
       <c r="AU145" s="1" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="146" spans="1:47">
@@ -24823,7 +24820,7 @@
         <v>270</v>
       </c>
       <c r="M146" s="1" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="N146" s="1" t="s">
         <v>291</v>
@@ -24862,34 +24859,34 @@
         <v>582</v>
       </c>
       <c r="AA146" s="1" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="AB146" s="1" t="s">
         <v>295</v>
       </c>
       <c r="AC146" s="1" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
       <c r="AD146" s="1" t="s">
         <v>347</v>
       </c>
       <c r="AE146" s="1" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="AF146" s="1" t="s">
-        <v>1073</v>
+        <v>1072</v>
       </c>
       <c r="AG146" s="1" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="AH146" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AI146" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AJ146" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK146" s="1" t="s">
         <v>318</v>
@@ -24922,7 +24919,7 @@
         <v>3</v>
       </c>
       <c r="AU146" s="1" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="147" spans="1:47">
@@ -24963,7 +24960,7 @@
         <v>270</v>
       </c>
       <c r="M147" s="1" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="N147" s="1" t="s">
         <v>291</v>
@@ -25002,13 +24999,13 @@
         <v>582</v>
       </c>
       <c r="AA147" s="1" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="AB147" s="1" t="s">
         <v>295</v>
       </c>
       <c r="AC147" s="1" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="AD147" s="1" t="s">
         <v>347</v>
@@ -25017,19 +25014,19 @@
         <v>348</v>
       </c>
       <c r="AF147" s="1" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="AG147" s="1" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="AH147" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AI147" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AJ147" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK147" s="1" t="s">
         <v>318</v>
@@ -25062,7 +25059,7 @@
         <v>3</v>
       </c>
       <c r="AU147" s="1" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="148" spans="1:47">
@@ -25130,7 +25127,7 @@
         <v>295</v>
       </c>
       <c r="W148" s="1" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="X148" s="1" t="s">
         <v>306</v>
@@ -25139,37 +25136,37 @@
         <v>307</v>
       </c>
       <c r="Z148" s="1" t="s">
+        <v>1065</v>
+      </c>
+      <c r="AA148" s="1" t="s">
         <v>1066</v>
-      </c>
-      <c r="AA148" s="1" t="s">
-        <v>1067</v>
       </c>
       <c r="AB148" s="1" t="s">
         <v>295</v>
       </c>
       <c r="AC148" s="1" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
       <c r="AD148" s="1" t="s">
         <v>347</v>
       </c>
       <c r="AE148" s="1" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="AF148" s="1" t="s">
+        <v>1072</v>
+      </c>
+      <c r="AG148" s="1" t="s">
         <v>1073</v>
       </c>
-      <c r="AG148" s="1" t="s">
-        <v>1074</v>
-      </c>
       <c r="AH148" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AI148" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AJ148" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK148" s="1" t="s">
         <v>318</v>
@@ -25202,7 +25199,7 @@
         <v>3</v>
       </c>
       <c r="AU148" s="1" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="149" spans="1:47">
@@ -25270,7 +25267,7 @@
         <v>295</v>
       </c>
       <c r="W149" s="1" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="X149" s="1" t="s">
         <v>306</v>
@@ -25279,37 +25276,37 @@
         <v>307</v>
       </c>
       <c r="Z149" s="1" t="s">
+        <v>1065</v>
+      </c>
+      <c r="AA149" s="1" t="s">
         <v>1066</v>
-      </c>
-      <c r="AA149" s="1" t="s">
-        <v>1067</v>
       </c>
       <c r="AB149" s="1" t="s">
         <v>295</v>
       </c>
       <c r="AC149" s="1" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="AD149" s="1" t="s">
         <v>347</v>
       </c>
       <c r="AE149" s="1" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="AF149" s="1" t="s">
+        <v>1081</v>
+      </c>
+      <c r="AG149" s="1" t="s">
+        <v>1075</v>
+      </c>
+      <c r="AH149" s="1" t="s">
         <v>1082</v>
       </c>
-      <c r="AG149" s="1" t="s">
-        <v>1076</v>
-      </c>
-      <c r="AH149" s="1" t="s">
-        <v>1083</v>
-      </c>
       <c r="AI149" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AJ149" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK149" s="1" t="s">
         <v>318</v>
@@ -25342,7 +25339,7 @@
         <v>3</v>
       </c>
       <c r="AU149" s="1" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="150" spans="1:47">
@@ -25410,7 +25407,7 @@
         <v>295</v>
       </c>
       <c r="W150" s="1" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="X150" s="1" t="s">
         <v>306</v>
@@ -25419,16 +25416,16 @@
         <v>307</v>
       </c>
       <c r="Z150" s="1" t="s">
+        <v>1065</v>
+      </c>
+      <c r="AA150" s="1" t="s">
         <v>1066</v>
-      </c>
-      <c r="AA150" s="1" t="s">
-        <v>1067</v>
       </c>
       <c r="AB150" s="1" t="s">
         <v>295</v>
       </c>
       <c r="AC150" s="1" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="AD150" s="1" t="s">
         <v>347</v>
@@ -25437,19 +25434,19 @@
         <v>348</v>
       </c>
       <c r="AF150" s="1" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="AG150" s="1" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="AH150" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AI150" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AJ150" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK150" s="1" t="s">
         <v>318</v>
@@ -25482,7 +25479,7 @@
         <v>3</v>
       </c>
       <c r="AU150" s="1" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="151" spans="1:47">
@@ -25550,7 +25547,7 @@
         <v>295</v>
       </c>
       <c r="W151" s="1" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="X151" s="1" t="s">
         <v>306</v>
@@ -25559,10 +25556,10 @@
         <v>307</v>
       </c>
       <c r="Z151" s="1" t="s">
+        <v>1065</v>
+      </c>
+      <c r="AA151" s="1" t="s">
         <v>1066</v>
-      </c>
-      <c r="AA151" s="1" t="s">
-        <v>1067</v>
       </c>
       <c r="AB151" s="1" t="s">
         <v>295</v>
@@ -25580,16 +25577,16 @@
         <v>842</v>
       </c>
       <c r="AG151" s="1" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="AH151" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AI151" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AJ151" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK151" s="1" t="s">
         <v>318</v>
@@ -25622,7 +25619,7 @@
         <v>3</v>
       </c>
       <c r="AU151" s="1" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="152" spans="1:47">
@@ -25663,7 +25660,7 @@
         <v>270</v>
       </c>
       <c r="M152" s="1" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="N152" s="1" t="s">
         <v>291</v>
@@ -25690,7 +25687,7 @@
         <v>295</v>
       </c>
       <c r="W152" s="1" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="X152" s="1" t="s">
         <v>306</v>
@@ -25699,37 +25696,37 @@
         <v>307</v>
       </c>
       <c r="Z152" s="1" t="s">
+        <v>1069</v>
+      </c>
+      <c r="AA152" s="1" t="s">
         <v>1070</v>
-      </c>
-      <c r="AA152" s="1" t="s">
-        <v>1071</v>
       </c>
       <c r="AB152" s="1" t="s">
         <v>295</v>
       </c>
       <c r="AC152" s="1" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
       <c r="AD152" s="1" t="s">
         <v>347</v>
       </c>
       <c r="AE152" s="1" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="AF152" s="1" t="s">
-        <v>1073</v>
+        <v>1072</v>
       </c>
       <c r="AG152" s="1" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="AH152" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AI152" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AJ152" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK152" s="1" t="s">
         <v>318</v>
@@ -25762,7 +25759,7 @@
         <v>3</v>
       </c>
       <c r="AU152" s="1" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="153" spans="1:47">
@@ -25803,7 +25800,7 @@
         <v>270</v>
       </c>
       <c r="M153" s="1" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="N153" s="1" t="s">
         <v>291</v>
@@ -25830,7 +25827,7 @@
         <v>295</v>
       </c>
       <c r="W153" s="1" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="X153" s="1" t="s">
         <v>306</v>
@@ -25839,16 +25836,16 @@
         <v>307</v>
       </c>
       <c r="Z153" s="1" t="s">
+        <v>1069</v>
+      </c>
+      <c r="AA153" s="1" t="s">
         <v>1070</v>
-      </c>
-      <c r="AA153" s="1" t="s">
-        <v>1071</v>
       </c>
       <c r="AB153" s="1" t="s">
         <v>295</v>
       </c>
       <c r="AC153" s="1" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="AD153" s="1" t="s">
         <v>347</v>
@@ -25857,19 +25854,19 @@
         <v>348</v>
       </c>
       <c r="AF153" s="1" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="AG153" s="1" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="AH153" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AI153" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="AJ153" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK153" s="1" t="s">
         <v>318</v>
@@ -25902,7 +25899,7 @@
         <v>3</v>
       </c>
       <c r="AU153" s="1" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="154" spans="1:47">
@@ -26250,7 +26247,7 @@
         <v>315</v>
       </c>
       <c r="U156" s="11" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="V156" s="1" t="s">
         <v>313</v>
@@ -26614,7 +26611,7 @@
         <v>10</v>
       </c>
       <c r="AU158" s="1" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
     </row>
     <row r="159" spans="1:47">
@@ -26757,12 +26754,12 @@
         <v>10</v>
       </c>
       <c r="AU159" s="1" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="160" spans="1:47">
       <c r="A160" s="1">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B160" s="1">
         <v>3</v>
@@ -26819,7 +26816,7 @@
         <v>336</v>
       </c>
       <c r="T160" s="11" t="s">
-        <v>931</v>
+        <v>578</v>
       </c>
       <c r="U160" s="11">
         <v>2005</v>
@@ -26900,12 +26897,12 @@
         <v>5</v>
       </c>
       <c r="AU160" s="1" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="161" spans="1:47">
       <c r="A161" s="1">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B161" s="11">
         <v>1</v>
@@ -26971,7 +26968,7 @@
         <v>295</v>
       </c>
       <c r="W161" s="11" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="X161" s="11" t="s">
         <v>879</v>
@@ -26980,10 +26977,10 @@
         <v>880</v>
       </c>
       <c r="Z161" s="11" t="s">
+        <v>1137</v>
+      </c>
+      <c r="AA161" s="11" t="s">
         <v>1138</v>
-      </c>
-      <c r="AA161" s="11" t="s">
-        <v>1139</v>
       </c>
       <c r="AB161" s="11" t="s">
         <v>345</v>
@@ -27010,10 +27007,10 @@
         <v>362</v>
       </c>
       <c r="AJ161" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="AK161" s="1" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="AL161" s="1" t="s">
         <v>315</v>
@@ -27043,7 +27040,7 @@
         <v>3</v>
       </c>
       <c r="AU161" s="1" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="162" spans="1:47">
@@ -27228,10 +27225,10 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="B1" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="C1" t="s">
         <v>318</v>
@@ -27240,7 +27237,7 @@
         <v>682</v>
       </c>
       <c r="E1" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -27390,12 +27387,12 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="D1" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="2" spans="1:20">
       <c r="D2" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -27405,66 +27402,66 @@
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="B4" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="C4" t="s">
         <v>683</v>
       </c>
       <c r="D4" t="s">
+        <v>1045</v>
+      </c>
+      <c r="E4" t="s">
         <v>1046</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
+        <v>1044</v>
+      </c>
+      <c r="G4" t="s">
+        <v>1002</v>
+      </c>
+      <c r="H4" t="s">
+        <v>1041</v>
+      </c>
+      <c r="I4" t="s">
+        <v>1040</v>
+      </c>
+      <c r="J4" t="s">
+        <v>1039</v>
+      </c>
+      <c r="K4" t="s">
+        <v>1049</v>
+      </c>
+      <c r="L4" t="s">
+        <v>1050</v>
+      </c>
+      <c r="M4" t="s">
+        <v>1048</v>
+      </c>
+      <c r="N4" t="s">
+        <v>1041</v>
+      </c>
+      <c r="O4" t="s">
         <v>1047</v>
       </c>
-      <c r="F4" t="s">
-        <v>1045</v>
-      </c>
-      <c r="G4" t="s">
-        <v>1003</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="P4" t="s">
         <v>1042</v>
-      </c>
-      <c r="I4" t="s">
-        <v>1041</v>
-      </c>
-      <c r="J4" t="s">
-        <v>1040</v>
-      </c>
-      <c r="K4" t="s">
-        <v>1050</v>
-      </c>
-      <c r="L4" t="s">
-        <v>1051</v>
-      </c>
-      <c r="M4" t="s">
-        <v>1049</v>
-      </c>
-      <c r="N4" t="s">
-        <v>1042</v>
-      </c>
-      <c r="O4" t="s">
-        <v>1048</v>
-      </c>
-      <c r="P4" t="s">
-        <v>1043</v>
       </c>
       <c r="R4" t="s">
         <v>319</v>
       </c>
       <c r="S4" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="T4" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="B5">
         <v>0.2</v>
@@ -27536,7 +27533,7 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B6">
         <v>0.04</v>
@@ -27566,7 +27563,7 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="B7">
         <v>0.05</v>
@@ -27624,7 +27621,7 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="B8">
         <v>0.11</v>
@@ -27657,30 +27654,30 @@
         <v>699</v>
       </c>
       <c r="B10" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="C10" t="s">
         <v>683</v>
       </c>
       <c r="D10" t="s">
+        <v>1045</v>
+      </c>
+      <c r="E10" t="s">
         <v>1046</v>
-      </c>
-      <c r="E10" t="s">
-        <v>1047</v>
       </c>
       <c r="R10" t="s">
         <v>320</v>
       </c>
       <c r="S10" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="T10" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="11" spans="1:20">
       <c r="A11" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="B11">
         <v>0.14000000000000001</v>
@@ -27752,7 +27749,7 @@
     </row>
     <row r="12" spans="1:20">
       <c r="A12" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="B12">
         <v>3.7999999999999999E-2</v>
@@ -27782,7 +27779,7 @@
     </row>
     <row r="13" spans="1:20">
       <c r="A13" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="B13">
         <v>0.17</v>
@@ -27840,7 +27837,7 @@
     </row>
     <row r="18" spans="1:20">
       <c r="A18" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="B18" t="s">
         <v>696</v>
@@ -27849,27 +27846,27 @@
         <v>683</v>
       </c>
       <c r="D18" t="s">
+        <v>1045</v>
+      </c>
+      <c r="E18" t="s">
         <v>1046</v>
       </c>
-      <c r="E18" t="s">
-        <v>1047</v>
-      </c>
       <c r="F18" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="R18" t="s">
         <v>319</v>
       </c>
       <c r="S18" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="T18" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="19" spans="1:20">
       <c r="A19" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="B19">
         <v>0.76</v>
@@ -27941,7 +27938,7 @@
     </row>
     <row r="20" spans="1:20">
       <c r="A20" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B20">
         <v>0.28999999999999998</v>
@@ -27971,7 +27968,7 @@
     </row>
     <row r="21" spans="1:20">
       <c r="A21" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="B21">
         <v>0.44</v>
@@ -28029,7 +28026,7 @@
     </row>
     <row r="22" spans="1:20">
       <c r="A22" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="B22">
         <v>0.49</v>
@@ -28062,33 +28059,33 @@
         <v>699</v>
       </c>
       <c r="B24" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="C24" t="s">
         <v>683</v>
       </c>
       <c r="D24" t="s">
+        <v>1045</v>
+      </c>
+      <c r="E24" t="s">
         <v>1046</v>
       </c>
-      <c r="E24" t="s">
-        <v>1047</v>
-      </c>
       <c r="F24" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="R24" t="s">
         <v>320</v>
       </c>
       <c r="S24" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="T24" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="25" spans="1:20">
       <c r="A25" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="B25">
         <v>0.82</v>
@@ -28160,7 +28157,7 @@
     </row>
     <row r="26" spans="1:20">
       <c r="A26" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="B26">
         <v>0.4</v>
@@ -28190,7 +28187,7 @@
     </row>
     <row r="27" spans="1:20">
       <c r="A27" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="B27">
         <v>0.39</v>
@@ -28437,7 +28434,7 @@
   <sheetData>
     <row r="1" spans="1:49" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -28584,7 +28581,7 @@
     </row>
     <row r="2" spans="1:49" s="1" customFormat="1">
       <c r="A2" s="1" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
@@ -28731,7 +28728,7 @@
     </row>
     <row r="3" spans="1:49" s="1" customFormat="1">
       <c r="A3" s="1" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="B3" s="1">
         <v>1</v>
@@ -28878,7 +28875,7 @@
     </row>
     <row r="4" spans="1:49" s="1" customFormat="1">
       <c r="A4" s="1" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="B4" s="1">
         <v>1</v>
@@ -29025,7 +29022,7 @@
     </row>
     <row r="5" spans="1:49" s="1" customFormat="1">
       <c r="A5" s="1" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="B5" s="1">
         <v>2</v>
@@ -29112,16 +29109,16 @@
         <v>313</v>
       </c>
       <c r="AD5" s="11" t="s">
+        <v>936</v>
+      </c>
+      <c r="AE5" s="11" t="s">
         <v>937</v>
       </c>
-      <c r="AE5" s="11" t="s">
+      <c r="AF5" s="11" t="s">
+        <v>959</v>
+      </c>
+      <c r="AG5" s="11" t="s">
         <v>938</v>
-      </c>
-      <c r="AF5" s="11" t="s">
-        <v>960</v>
-      </c>
-      <c r="AG5" s="11" t="s">
-        <v>939</v>
       </c>
       <c r="AH5" s="11" t="s">
         <v>923</v>
@@ -29167,12 +29164,12 @@
       </c>
       <c r="AV5"/>
       <c r="AW5" s="11" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
     </row>
     <row r="6" spans="1:49" s="1" customFormat="1">
       <c r="A6" s="1" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="B6" s="1">
         <v>2</v>
@@ -29259,16 +29256,16 @@
         <v>313</v>
       </c>
       <c r="AD6" s="11" t="s">
+        <v>936</v>
+      </c>
+      <c r="AE6" s="11" t="s">
         <v>937</v>
       </c>
-      <c r="AE6" s="11" t="s">
+      <c r="AF6" s="11" t="s">
+        <v>959</v>
+      </c>
+      <c r="AG6" s="11" t="s">
         <v>938</v>
-      </c>
-      <c r="AF6" s="11" t="s">
-        <v>960</v>
-      </c>
-      <c r="AG6" s="11" t="s">
-        <v>939</v>
       </c>
       <c r="AH6" s="11" t="s">
         <v>923</v>
@@ -29319,7 +29316,7 @@
     </row>
     <row r="7" spans="1:49" s="1" customFormat="1">
       <c r="A7" s="1" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="B7" s="1">
         <v>2</v>
@@ -29430,7 +29427,7 @@
         <v>800</v>
       </c>
       <c r="AL7" s="1" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="AM7" s="11" t="s">
         <v>315</v>
@@ -29466,7 +29463,7 @@
     </row>
     <row r="8" spans="1:49" s="1" customFormat="1">
       <c r="A8" s="1" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="B8" s="1">
         <v>2</v>
@@ -29529,7 +29526,7 @@
         <v>578</v>
       </c>
       <c r="V8" s="5" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="W8" s="1" t="s">
         <v>295</v>
@@ -29553,22 +29550,22 @@
         <v>313</v>
       </c>
       <c r="AD8" s="11" t="s">
+        <v>936</v>
+      </c>
+      <c r="AE8" s="11" t="s">
         <v>937</v>
       </c>
-      <c r="AE8" s="11" t="s">
+      <c r="AF8" s="11" t="s">
+        <v>959</v>
+      </c>
+      <c r="AG8" s="11" t="s">
         <v>938</v>
-      </c>
-      <c r="AF8" s="11" t="s">
-        <v>960</v>
-      </c>
-      <c r="AG8" s="11" t="s">
-        <v>939</v>
       </c>
       <c r="AH8" s="11" t="s">
         <v>923</v>
       </c>
       <c r="AI8" s="11" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="AJ8" s="11" t="s">
         <v>362</v>
@@ -29608,12 +29605,12 @@
       </c>
       <c r="AV8"/>
       <c r="AW8" s="1" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
     </row>
     <row r="9" spans="1:49" s="1" customFormat="1">
       <c r="A9" s="1" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="B9" s="1">
         <v>2</v>
@@ -29698,22 +29695,22 @@
         <v>313</v>
       </c>
       <c r="AD9" s="11" t="s">
+        <v>936</v>
+      </c>
+      <c r="AE9" s="11" t="s">
         <v>937</v>
       </c>
-      <c r="AE9" s="11" t="s">
+      <c r="AF9" s="11" t="s">
+        <v>959</v>
+      </c>
+      <c r="AG9" s="11" t="s">
         <v>938</v>
-      </c>
-      <c r="AF9" s="11" t="s">
-        <v>960</v>
-      </c>
-      <c r="AG9" s="11" t="s">
-        <v>939</v>
       </c>
       <c r="AH9" s="11" t="s">
         <v>923</v>
       </c>
       <c r="AI9" s="11" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="AJ9" s="11" t="s">
         <v>362</v>
@@ -29753,12 +29750,12 @@
       </c>
       <c r="AV9"/>
       <c r="AW9" s="1" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
     </row>
     <row r="10" spans="1:49" s="1" customFormat="1">
       <c r="A10" s="1" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="B10" s="1">
         <v>2</v>
@@ -29858,7 +29855,7 @@
         <v>898</v>
       </c>
       <c r="AI10" s="11" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="AJ10" s="11" t="s">
         <v>362</v>
@@ -29867,7 +29864,7 @@
         <v>800</v>
       </c>
       <c r="AL10" s="11" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="AM10" s="11" t="s">
         <v>315</v>
@@ -29898,12 +29895,12 @@
       </c>
       <c r="AV10"/>
       <c r="AW10" s="1" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
     </row>
     <row r="11" spans="1:49" s="1" customFormat="1">
       <c r="A11" s="1" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="B11" s="1">
         <v>2</v>
@@ -30003,7 +30000,7 @@
         <v>898</v>
       </c>
       <c r="AI11" s="11" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="AJ11" s="11" t="s">
         <v>362</v>
@@ -30043,12 +30040,12 @@
       </c>
       <c r="AV11"/>
       <c r="AW11" s="1" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
     </row>
     <row r="12" spans="1:49" s="1" customFormat="1">
       <c r="A12" s="1" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="B12" s="1">
         <v>3</v>
@@ -30099,7 +30096,7 @@
         <v>424</v>
       </c>
       <c r="R12" s="1" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="S12" s="1" t="s">
         <v>315</v>
@@ -30111,7 +30108,7 @@
         <v>315</v>
       </c>
       <c r="V12" s="1" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="W12" s="1" t="s">
         <v>295</v>
@@ -30126,16 +30123,16 @@
         <v>581</v>
       </c>
       <c r="AA12" s="1" t="s">
+        <v>974</v>
+      </c>
+      <c r="AB12" s="1" t="s">
         <v>975</v>
-      </c>
-      <c r="AB12" s="1" t="s">
-        <v>976</v>
       </c>
       <c r="AC12" s="1" t="s">
         <v>295</v>
       </c>
       <c r="AD12" s="1" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="AE12" s="1" t="s">
         <v>662</v>
@@ -30144,10 +30141,10 @@
         <v>601</v>
       </c>
       <c r="AG12" s="1" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="AH12" s="1" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="AI12" s="1" t="s">
         <v>829</v>
@@ -30159,7 +30156,7 @@
         <v>746</v>
       </c>
       <c r="AL12" s="1" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="AM12" s="1" t="s">
         <v>315</v>
@@ -30190,12 +30187,12 @@
       </c>
       <c r="AV12"/>
       <c r="AW12" s="1" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
     </row>
     <row r="13" spans="1:49" s="1" customFormat="1">
       <c r="A13" s="1" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="B13" s="1">
         <v>3</v>
@@ -30246,7 +30243,7 @@
         <v>424</v>
       </c>
       <c r="R13" s="1" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="S13" s="1" t="s">
         <v>315</v>
@@ -30258,7 +30255,7 @@
         <v>315</v>
       </c>
       <c r="V13" s="1" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="W13" s="1" t="s">
         <v>295</v>
@@ -30273,16 +30270,16 @@
         <v>581</v>
       </c>
       <c r="AA13" s="1" t="s">
+        <v>974</v>
+      </c>
+      <c r="AB13" s="1" t="s">
         <v>975</v>
-      </c>
-      <c r="AB13" s="1" t="s">
-        <v>976</v>
       </c>
       <c r="AC13" s="1" t="s">
         <v>295</v>
       </c>
       <c r="AD13" s="1" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="AE13" s="1" t="s">
         <v>662</v>
@@ -30291,10 +30288,10 @@
         <v>601</v>
       </c>
       <c r="AG13" s="1" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="AH13" s="1" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="AI13" s="1" t="s">
         <v>732</v>
@@ -30306,7 +30303,7 @@
         <v>746</v>
       </c>
       <c r="AL13" s="1" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="AM13" s="1" t="s">
         <v>315</v>
@@ -30337,7 +30334,7 @@
       </c>
       <c r="AV13"/>
       <c r="AW13" s="1" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
     </row>
   </sheetData>
@@ -30475,7 +30472,7 @@
         <v>586</v>
       </c>
       <c r="AP1" s="1" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="AQ1" s="1" t="s">
         <v>320</v>
@@ -30531,7 +30528,7 @@
         <v>272</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="N2" s="1" t="s">
         <v>291</v>
@@ -30563,10 +30560,10 @@
         <v>1998</v>
       </c>
       <c r="G3" s="1" t="s">
+        <v>1143</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>1144</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>1145</v>
       </c>
       <c r="I3" s="1">
         <v>-36.306666999999997</v>
@@ -30578,7 +30575,7 @@
         <v>371</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="M3" s="1" t="s">
         <v>645</v>
@@ -30613,10 +30610,10 @@
         <v>1985</v>
       </c>
       <c r="G4" s="1" t="s">
+        <v>1146</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>1147</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>1148</v>
       </c>
       <c r="I4" s="1">
         <v>17.758092999999999</v>
@@ -30628,7 +30625,7 @@
         <v>366</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="M4" s="1" t="s">
         <v>574</v>
@@ -30663,10 +30660,10 @@
         <v>2018</v>
       </c>
       <c r="G5" s="1" t="s">
+        <v>1150</v>
+      </c>
+      <c r="H5" s="1" t="s">
         <v>1151</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>1152</v>
       </c>
       <c r="I5" s="1">
         <v>33.587860999999997</v>
@@ -30678,7 +30675,7 @@
         <v>366</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="M5" s="1" t="s">
         <v>574</v>
@@ -30713,10 +30710,10 @@
         <v>2018</v>
       </c>
       <c r="G6" s="1" t="s">
+        <v>1152</v>
+      </c>
+      <c r="H6" s="1" t="s">
         <v>1153</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>1154</v>
       </c>
       <c r="I6" s="1">
         <v>-5.8333329999999997</v>
@@ -30725,7 +30722,7 @@
         <v>72</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
       <c r="L6" s="1" t="s">
         <v>380</v>
@@ -30763,10 +30760,10 @@
         <v>2017</v>
       </c>
       <c r="G7" s="1" t="s">
+        <v>1155</v>
+      </c>
+      <c r="H7" s="1" t="s">
         <v>1156</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>1157</v>
       </c>
       <c r="I7" s="1">
         <v>29.469228999999999</v>
@@ -30813,10 +30810,10 @@
         <v>2014</v>
       </c>
       <c r="G8" s="1" t="s">
+        <v>1157</v>
+      </c>
+      <c r="H8" s="1" t="s">
         <v>1158</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>1159</v>
       </c>
       <c r="I8" s="1">
         <v>24.095333</v>
@@ -30828,7 +30825,7 @@
         <v>363</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="M8" s="1" t="s">
         <v>574</v>
@@ -30863,10 +30860,10 @@
         <v>2014</v>
       </c>
       <c r="G9" s="1" t="s">
+        <v>1160</v>
+      </c>
+      <c r="H9" s="1" t="s">
         <v>1161</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>1162</v>
       </c>
       <c r="I9" s="1">
         <v>42.224753999999997</v>
@@ -30875,7 +30872,7 @@
         <v>-8.8175150000000002</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="P9" s="1" t="s">
         <v>338</v>
@@ -30901,10 +30898,10 @@
         <v>2011</v>
       </c>
       <c r="G10" s="1" t="s">
+        <v>1162</v>
+      </c>
+      <c r="H10" s="1" t="s">
         <v>1163</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>1164</v>
       </c>
       <c r="I10" s="1">
         <v>-45.691389000000001</v>
@@ -30939,10 +30936,10 @@
         <v>2011</v>
       </c>
       <c r="G11" s="1" t="s">
+        <v>1165</v>
+      </c>
+      <c r="H11" s="1" t="s">
         <v>1166</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>1167</v>
       </c>
       <c r="I11" s="1">
         <v>-53.244253</v>
@@ -30951,7 +30948,7 @@
         <v>-37.673316</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="P11" s="1" t="s">
         <v>276</v>
@@ -30977,10 +30974,10 @@
         <v>2007</v>
       </c>
       <c r="G12" s="1" t="s">
+        <v>1168</v>
+      </c>
+      <c r="H12" s="1" t="s">
         <v>1169</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>1170</v>
       </c>
       <c r="I12" s="1">
         <v>38.315517999999997</v>
@@ -31015,10 +31012,10 @@
         <v>2006</v>
       </c>
       <c r="G13" s="1" t="s">
+        <v>1170</v>
+      </c>
+      <c r="H13" s="1" t="s">
         <v>1171</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>1172</v>
       </c>
       <c r="I13" s="1">
         <v>-45.783529999999999</v>
@@ -31053,10 +31050,10 @@
         <v>2004</v>
       </c>
       <c r="G14" s="1" t="s">
+        <v>1172</v>
+      </c>
+      <c r="H14" s="1" t="s">
         <v>1173</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>1174</v>
       </c>
       <c r="I14" s="1">
         <v>44.255260999999997</v>
@@ -31091,10 +31088,10 @@
         <v>2000</v>
       </c>
       <c r="G15" s="1" t="s">
+        <v>1175</v>
+      </c>
+      <c r="H15" s="1" t="s">
         <v>1176</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>1177</v>
       </c>
       <c r="I15" s="1">
         <v>34.259346999999998</v>
@@ -31103,7 +31100,7 @@
         <v>133.40153699999999</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="P15" s="1" t="s">
         <v>424</v>
@@ -31129,10 +31126,10 @@
         <v>2000</v>
       </c>
       <c r="G16" s="1" t="s">
+        <v>1177</v>
+      </c>
+      <c r="H16" s="1" t="s">
         <v>1178</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>1179</v>
       </c>
       <c r="I16" s="1">
         <v>-34.112057</v>
@@ -31167,10 +31164,10 @@
         <v>1999</v>
       </c>
       <c r="G17" s="1" t="s">
+        <v>1179</v>
+      </c>
+      <c r="H17" s="1" t="s">
         <v>1180</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>1181</v>
       </c>
       <c r="I17" s="1">
         <v>30.5</v>
@@ -31205,10 +31202,10 @@
         <v>1998</v>
       </c>
       <c r="G18" s="1" t="s">
+        <v>1181</v>
+      </c>
+      <c r="H18" s="1" t="s">
         <v>1182</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>1183</v>
       </c>
       <c r="I18" s="1">
         <v>29.096662999999999</v>
@@ -31243,10 +31240,10 @@
         <v>1994</v>
       </c>
       <c r="G19" s="1" t="s">
+        <v>1183</v>
+      </c>
+      <c r="H19" s="1" t="s">
         <v>1184</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>1185</v>
       </c>
       <c r="I19" s="1">
         <v>48.853999999999999</v>
@@ -31281,10 +31278,10 @@
         <v>2010</v>
       </c>
       <c r="G20" s="1" t="s">
+        <v>1185</v>
+      </c>
+      <c r="H20" s="1" t="s">
         <v>1186</v>
-      </c>
-      <c r="H20" s="1" t="s">
-        <v>1187</v>
       </c>
       <c r="I20" s="1">
         <v>54.35</v>
@@ -31293,7 +31290,7 @@
         <v>10.15</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="P20" s="1" t="s">
         <v>338</v>
@@ -31319,10 +31316,10 @@
         <v>1998</v>
       </c>
       <c r="G21" s="1" t="s">
+        <v>1188</v>
+      </c>
+      <c r="H21" s="1" t="s">
         <v>1189</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>1190</v>
       </c>
       <c r="I21" s="1">
         <v>-63.134332999999998</v>
@@ -31331,7 +31328,7 @@
         <v>-51.091971999999998</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="P21" s="1" t="s">
         <v>276</v>
@@ -31357,10 +31354,10 @@
         <v>1993</v>
       </c>
       <c r="G22" s="1" t="s">
+        <v>1190</v>
+      </c>
+      <c r="H22" s="1" t="s">
         <v>1191</v>
-      </c>
-      <c r="H22" s="1" t="s">
-        <v>1192</v>
       </c>
       <c r="I22" s="1">
         <v>58.866667</v>
@@ -31369,7 +31366,7 @@
         <v>11.15</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="P22" s="1" t="s">
         <v>338</v>
@@ -31395,10 +31392,10 @@
         <v>1988</v>
       </c>
       <c r="G23" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="H23" s="1" t="s">
         <v>1194</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>1195</v>
       </c>
       <c r="I23" s="1">
         <v>33.466667000000001</v>
@@ -31433,10 +31430,10 @@
         <v>1982</v>
       </c>
       <c r="G24" s="1" t="s">
+        <v>1195</v>
+      </c>
+      <c r="H24" s="1" t="s">
         <v>1196</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>1197</v>
       </c>
       <c r="I24" s="1">
         <v>41.588000000000001</v>
@@ -31585,7 +31582,7 @@
     </row>
     <row r="28" spans="1:49" s="1" customFormat="1">
       <c r="A28" s="1" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="B28" s="1">
         <v>27</v>
@@ -31639,10 +31636,10 @@
         <v>581</v>
       </c>
       <c r="AA28" s="1" t="s">
+        <v>1056</v>
+      </c>
+      <c r="AB28" s="1" t="s">
         <v>1057</v>
-      </c>
-      <c r="AB28" s="1" t="s">
-        <v>1058</v>
       </c>
       <c r="AC28" s="1" t="s">
         <v>295</v>
@@ -31650,7 +31647,7 @@
     </row>
     <row r="29" spans="1:49" s="1" customFormat="1">
       <c r="A29" s="1" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
       <c r="B29" s="1">
         <v>28</v>
@@ -31668,10 +31665,10 @@
         <v>2013</v>
       </c>
       <c r="G29" s="1" t="s">
+        <v>1133</v>
+      </c>
+      <c r="H29" s="1" t="s">
         <v>1134</v>
-      </c>
-      <c r="H29" s="1" t="s">
-        <v>1135</v>
       </c>
       <c r="I29" s="1">
         <v>25.0349</v>
@@ -31719,7 +31716,7 @@
     </row>
     <row r="30" spans="1:49" s="1" customFormat="1">
       <c r="A30" s="1" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
       <c r="B30" s="1">
         <v>29</v>
@@ -31905,7 +31902,7 @@
         <v>586</v>
       </c>
       <c r="AP1" s="1" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="AQ1" s="1" t="s">
         <v>320</v>
@@ -32095,7 +32092,7 @@
     </row>
     <row r="12" spans="1:47" s="1" customFormat="1">
       <c r="A12" s="1" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>195</v>
@@ -32441,7 +32438,7 @@
     </row>
     <row r="26" spans="1:49" s="1" customFormat="1">
       <c r="A26" s="1" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="B26" s="11">
         <v>1</v>
@@ -32489,7 +32486,7 @@
         <v>338</v>
       </c>
       <c r="Q26" s="1" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="R26" s="1" t="s">
         <v>315</v>
@@ -32507,7 +32504,7 @@
         <v>313</v>
       </c>
       <c r="W26" s="1" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="X26" s="1" t="s">
         <v>885</v>
@@ -32516,7 +32513,7 @@
         <v>886</v>
       </c>
       <c r="Z26" s="1" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="AA26" s="1" t="s">
         <v>923</v>
@@ -32524,7 +32521,7 @@
     </row>
     <row r="27" spans="1:49" s="1" customFormat="1">
       <c r="A27" s="1" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="B27" s="11">
         <v>1</v>
@@ -32572,7 +32569,7 @@
         <v>425</v>
       </c>
       <c r="Q27" s="1" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="R27" s="1" t="s">
         <v>315</v>
@@ -32590,7 +32587,7 @@
         <v>295</v>
       </c>
       <c r="W27" s="1" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="X27" s="1" t="s">
         <v>885</v>
@@ -32599,14 +32596,14 @@
         <v>886</v>
       </c>
       <c r="Z27" s="1" t="s">
+        <v>1023</v>
+      </c>
+      <c r="AA27" s="1" t="s">
         <v>1024</v>
-      </c>
-      <c r="AA27" s="1" t="s">
-        <v>1025</v>
       </c>
       <c r="AV27"/>
       <c r="AW27" s="1" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
     </row>
     <row r="28" spans="1:49" s="1" customFormat="1">
@@ -32718,7 +32715,7 @@
       </c>
       <c r="E1" s="3"/>
       <c r="F1" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -32726,7 +32723,7 @@
         <v>420</v>
       </c>
       <c r="F2" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -32734,7 +32731,7 @@
         <v>421</v>
       </c>
       <c r="F3" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -32829,7 +32826,7 @@
     </row>
     <row r="27" spans="1:1">
       <c r="A27" s="4" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
     </row>
   </sheetData>
@@ -32847,10 +32844,10 @@
   <sheetData>
     <row r="1" spans="2:10">
       <c r="B1" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="E1" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="G1" t="s">
         <v>865</v>
@@ -32861,7 +32858,7 @@
         <v>682</v>
       </c>
       <c r="C2" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="D2" t="s">
         <v>683</v>
@@ -32870,7 +32867,7 @@
         <v>682</v>
       </c>
       <c r="H2" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="I2" t="s">
         <v>683</v>
@@ -33223,7 +33220,7 @@
         <v>586</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>320</v>
@@ -33866,7 +33863,7 @@
     </row>
     <row r="23" spans="1:13">
       <c r="A23" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
     </row>
     <row r="24" spans="1:13">
@@ -34013,7 +34010,7 @@
     </row>
     <row r="35" spans="1:16">
       <c r="A35" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
     </row>
     <row r="36" spans="1:16">
@@ -34082,7 +34079,7 @@
     </row>
     <row r="41" spans="1:16">
       <c r="A41" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="C41" t="s">
         <v>682</v>
@@ -34146,10 +34143,10 @@
     </row>
     <row r="45" spans="1:16">
       <c r="A45" s="10" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="J45" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
     </row>
     <row r="46" spans="1:16">
@@ -34157,7 +34154,7 @@
         <v>350</v>
       </c>
       <c r="B46" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="J46" t="s">
         <v>350</v>
@@ -34287,7 +34284,7 @@
     </row>
     <row r="52" spans="1:16">
       <c r="A52" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="C52" t="s">
         <v>682</v>
@@ -34305,7 +34302,7 @@
         <v>736</v>
       </c>
       <c r="J52" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="L52" t="s">
         <v>682</v>
@@ -34409,10 +34406,10 @@
     </row>
     <row r="56" spans="1:16">
       <c r="A56" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="J56" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
     </row>
     <row r="57" spans="1:16">
@@ -34539,7 +34536,7 @@
     </row>
     <row r="62" spans="1:16">
       <c r="A62" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="C62" t="s">
         <v>682</v>
@@ -34557,7 +34554,7 @@
         <v>736</v>
       </c>
       <c r="J62" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="L62" t="s">
         <v>682</v>
@@ -34661,10 +34658,10 @@
     </row>
     <row r="66" spans="1:16">
       <c r="A66" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="J66" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
     <row r="67" spans="1:16">
@@ -34791,7 +34788,7 @@
     </row>
     <row r="72" spans="1:16">
       <c r="A72" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="C72" t="s">
         <v>682</v>
@@ -34809,7 +34806,7 @@
         <v>736</v>
       </c>
       <c r="J72" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="L72" t="s">
         <v>682</v>
@@ -34913,10 +34910,10 @@
     </row>
     <row r="76" spans="1:16">
       <c r="A76" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="J76" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
     </row>
     <row r="77" spans="1:16">
@@ -35043,7 +35040,7 @@
     </row>
     <row r="82" spans="1:16">
       <c r="A82" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="C82" t="s">
         <v>682</v>
@@ -35061,7 +35058,7 @@
         <v>736</v>
       </c>
       <c r="J82" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="L82" t="s">
         <v>682</v>
@@ -35165,7 +35162,7 @@
     </row>
     <row r="86" spans="1:16">
       <c r="A86" s="10" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
     </row>
     <row r="87" spans="1:16">
@@ -35239,7 +35236,7 @@
     </row>
     <row r="93" spans="1:16">
       <c r="A93" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="C93" t="s">
         <v>682</v>
@@ -35372,7 +35369,7 @@
     </row>
     <row r="103" spans="1:7">
       <c r="A103" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="C103" t="s">
         <v>682</v>
@@ -35532,7 +35529,7 @@
     </row>
     <row r="113" spans="1:7">
       <c r="A113" s="7" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="B113" s="7"/>
       <c r="C113" s="7" t="s">
@@ -35599,7 +35596,7 @@
     </row>
     <row r="118" spans="1:7">
       <c r="A118" s="10" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="120" spans="1:7">
@@ -35689,7 +35686,7 @@
     </row>
     <row r="125" spans="1:7">
       <c r="A125" s="7" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="B125" s="7"/>
       <c r="C125" s="7" t="s">
@@ -35756,12 +35753,12 @@
     </row>
     <row r="130" spans="1:7">
       <c r="A130" s="10" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="132" spans="1:7">
       <c r="A132" s="7" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="B132" s="7"/>
       <c r="C132" s="7" t="s">
@@ -35846,7 +35843,7 @@
     </row>
     <row r="137" spans="1:7">
       <c r="A137" s="7" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="B137" s="7"/>
       <c r="C137" s="7" t="s">
@@ -35913,12 +35910,12 @@
     </row>
     <row r="142" spans="1:7">
       <c r="A142" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="144" spans="1:7">
       <c r="A144" s="7" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="B144" s="7"/>
       <c r="C144" s="7" t="s">
@@ -36003,7 +36000,7 @@
     </row>
     <row r="149" spans="1:7">
       <c r="A149" s="7" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="B149" s="7"/>
       <c r="C149" s="7" t="s">
@@ -36090,7 +36087,7 @@
     </row>
     <row r="6" spans="1:13">
       <c r="A6" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -36869,7 +36866,7 @@
     </row>
     <row r="45" spans="1:9">
       <c r="A45" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -36972,35 +36969,35 @@
     </row>
     <row r="52" spans="1:10">
       <c r="A52" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="53" spans="1:10">
       <c r="D53" t="s">
+        <v>1093</v>
+      </c>
+      <c r="E53" t="s">
+        <v>1092</v>
+      </c>
+      <c r="F53" t="s">
+        <v>1095</v>
+      </c>
+      <c r="H53" t="s">
         <v>1094</v>
       </c>
-      <c r="E53" t="s">
-        <v>1093</v>
-      </c>
-      <c r="F53" t="s">
+      <c r="I53" t="s">
+        <v>1092</v>
+      </c>
+      <c r="J53" t="s">
         <v>1096</v>
-      </c>
-      <c r="H53" t="s">
-        <v>1095</v>
-      </c>
-      <c r="I53" t="s">
-        <v>1093</v>
-      </c>
-      <c r="J53" t="s">
-        <v>1097</v>
       </c>
     </row>
     <row r="54" spans="1:10">
       <c r="A54" t="s">
+        <v>1084</v>
+      </c>
+      <c r="C54" t="s">
         <v>1085</v>
-      </c>
-      <c r="C54" t="s">
-        <v>1086</v>
       </c>
       <c r="D54">
         <v>0.35</v>
@@ -37025,7 +37022,7 @@
     </row>
     <row r="55" spans="1:10">
       <c r="C55" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="D55">
         <v>0.49</v>
@@ -37050,7 +37047,7 @@
     </row>
     <row r="56" spans="1:10">
       <c r="C56" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="D56">
         <v>0.46</v>
@@ -37075,7 +37072,7 @@
     </row>
     <row r="57" spans="1:10">
       <c r="C57" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
       <c r="D57">
         <v>0.96</v>
@@ -37103,7 +37100,7 @@
         <v>746</v>
       </c>
       <c r="C59" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
       <c r="D59">
         <v>0.43</v>
@@ -37128,7 +37125,7 @@
     </row>
     <row r="60" spans="1:10">
       <c r="C60" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="D60">
         <v>1.63</v>
@@ -37153,11 +37150,11 @@
     </row>
     <row r="62" spans="1:10">
       <c r="A62" s="7" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="B62" s="7"/>
       <c r="C62" s="7" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D62">
         <v>0.35</v>
@@ -37184,7 +37181,7 @@
       <c r="A63" s="7"/>
       <c r="B63" s="7"/>
       <c r="C63" s="7" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="D63">
         <v>0.42</v>
@@ -37211,7 +37208,7 @@
       <c r="A64" s="7"/>
       <c r="B64" s="7"/>
       <c r="C64" s="7" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="D64">
         <v>0</v>
@@ -37238,7 +37235,7 @@
       <c r="A65" s="7"/>
       <c r="B65" s="7"/>
       <c r="C65" s="7" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
       <c r="D65">
         <v>0.28999999999999998</v>
@@ -37263,11 +37260,11 @@
     </row>
     <row r="67" spans="1:10">
       <c r="A67" s="7" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
       <c r="B67" s="7"/>
       <c r="C67" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
       <c r="D67">
         <v>0.28999999999999998</v>
@@ -37294,7 +37291,7 @@
       <c r="A68" s="7"/>
       <c r="B68" s="7"/>
       <c r="C68" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="D68">
         <v>0.15</v>
@@ -37329,24 +37326,24 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" t="s">
+        <v>997</v>
+      </c>
+      <c r="B1" t="s">
         <v>998</v>
       </c>
-      <c r="B1" t="s">
-        <v>999</v>
-      </c>
       <c r="R1" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="S1" t="s">
         <v>682</v>
       </c>
       <c r="T1" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
     </row>
     <row r="2" spans="1:20">
       <c r="B2" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="C2">
         <v>0.42857142857142799</v>
@@ -37445,7 +37442,7 @@
     </row>
     <row r="5" spans="1:20">
       <c r="B5" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="C5">
         <v>0.22396313364055201</v>
@@ -37503,10 +37500,10 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="B8" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="C8">
         <v>0.29308755760368599</v>
@@ -37653,7 +37650,7 @@
     </row>
     <row r="11" spans="1:20">
       <c r="B11" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="C11">
         <v>0.31244239631336301</v>
@@ -37750,7 +37747,7 @@
         <v>586</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>320</v>

</xml_diff>

<commit_message>
updated dfs with the 2 new papers
</commit_message>
<xml_diff>
--- a/Output/Data/meta_analysis_data.xlsx
+++ b/Output/Data/meta_analysis_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilylim/Documents/MSc/Ch2-Meta-analysis/Output/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{929B4D3E-53F9-BB40-B812-4CEFF04A2FD0}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46E8F86A-FAEF-804C-AA6E-D6028D63EFBF}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10700" yWindow="460" windowWidth="19600" windowHeight="15940" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
+    <workbookView xWindow="9200" yWindow="460" windowWidth="19600" windowHeight="15840" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
   </bookViews>
   <sheets>
     <sheet name="Include" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
updated coordinates for peterson paper
</commit_message>
<xml_diff>
--- a/Output/Data/meta_analysis_data.xlsx
+++ b/Output/Data/meta_analysis_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilylim/Documents/MSc/Ch2-Meta-analysis/Output/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6014E838-D7CC-8F49-8BD3-FB52D40FAA1C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F651994A-96A8-7E4D-A8F7-A42A790DD72B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9520" yWindow="460" windowWidth="27540" windowHeight="18740" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
+    <workbookView xWindow="6560" yWindow="460" windowWidth="27540" windowHeight="15860" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
   </bookViews>
   <sheets>
     <sheet name="Include" sheetId="1" r:id="rId1"/>
@@ -20357,11 +20357,11 @@
       <c r="I107" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="J107" s="1">
-        <v>29.770776999999999</v>
-      </c>
-      <c r="K107" s="1">
-        <v>-85.357286000000002</v>
+      <c r="J107">
+        <v>29.704194999999999</v>
+      </c>
+      <c r="K107">
+        <v>-85.469155999999998</v>
       </c>
       <c r="L107" s="1" t="s">
         <v>365</v>
@@ -20506,11 +20506,11 @@
       <c r="I108" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="J108" s="1">
-        <v>29.770776999999999</v>
-      </c>
-      <c r="K108" s="1">
-        <v>-85.357286000000002</v>
+      <c r="J108">
+        <v>29.704194999999999</v>
+      </c>
+      <c r="K108">
+        <v>-85.469155999999998</v>
       </c>
       <c r="L108" s="1" t="s">
         <v>365</v>
@@ -20655,11 +20655,11 @@
       <c r="I109" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="J109" s="1">
-        <v>29.770776999999999</v>
-      </c>
-      <c r="K109" s="1">
-        <v>-85.357286000000002</v>
+      <c r="J109">
+        <v>29.704194999999999</v>
+      </c>
+      <c r="K109">
+        <v>-85.469155999999998</v>
       </c>
       <c r="L109" s="1" t="s">
         <v>365</v>
@@ -20804,11 +20804,11 @@
       <c r="I110" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="J110" s="1">
-        <v>29.770776999999999</v>
-      </c>
-      <c r="K110" s="1">
-        <v>-85.357286000000002</v>
+      <c r="J110">
+        <v>29.704194999999999</v>
+      </c>
+      <c r="K110">
+        <v>-85.469155999999998</v>
       </c>
       <c r="L110" s="1" t="s">
         <v>365</v>
@@ -20953,11 +20953,11 @@
       <c r="I111" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="J111" s="1">
-        <v>29.770776999999999</v>
-      </c>
-      <c r="K111" s="1">
-        <v>-85.357286000000002</v>
+      <c r="J111">
+        <v>29.704194999999999</v>
+      </c>
+      <c r="K111">
+        <v>-85.469155999999998</v>
       </c>
       <c r="L111" s="1" t="s">
         <v>365</v>
@@ -21102,11 +21102,11 @@
       <c r="I112" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="J112" s="1">
-        <v>29.770776999999999</v>
-      </c>
-      <c r="K112" s="1">
-        <v>-85.357286000000002</v>
+      <c r="J112">
+        <v>29.704194999999999</v>
+      </c>
+      <c r="K112">
+        <v>-85.469155999999998</v>
       </c>
       <c r="L112" s="1" t="s">
         <v>365</v>
@@ -21251,11 +21251,11 @@
       <c r="I113" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="J113" s="1">
-        <v>29.770776999999999</v>
-      </c>
-      <c r="K113" s="1">
-        <v>-85.357286000000002</v>
+      <c r="J113">
+        <v>29.704194999999999</v>
+      </c>
+      <c r="K113">
+        <v>-85.469155999999998</v>
       </c>
       <c r="L113" s="1" t="s">
         <v>365</v>
@@ -21400,11 +21400,11 @@
       <c r="I114" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="J114" s="1">
-        <v>29.770776999999999</v>
-      </c>
-      <c r="K114" s="1">
-        <v>-85.357286000000002</v>
+      <c r="J114">
+        <v>29.704194999999999</v>
+      </c>
+      <c r="K114">
+        <v>-85.469155999999998</v>
       </c>
       <c r="L114" s="1" t="s">
         <v>365</v>

</xml_diff>

<commit_message>
change the one mangrove pp_taxa from NA to O
</commit_message>
<xml_diff>
--- a/Output/Data/meta_analysis_data.xlsx
+++ b/Output/Data/meta_analysis_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilylim/Documents/MSc/Ch2-Meta-analysis/Output/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9389781A-99F2-8648-AA41-EC64839987E3}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{965E1AE5-D7BA-F049-8728-EE034CCC1698}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="880" yWindow="460" windowWidth="27540" windowHeight="15860" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
   </bookViews>
@@ -30091,7 +30091,7 @@
         <v>880</v>
       </c>
       <c r="AF172" s="11" t="s">
-        <v>314</v>
+        <v>656</v>
       </c>
       <c r="AG172" s="11" t="s">
         <v>596</v>

</xml_diff>

<commit_message>
i think there was a typo in one of the lines
</commit_message>
<xml_diff>
--- a/Output/Data/meta_analysis_data.xlsx
+++ b/Output/Data/meta_analysis_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilylim/Documents/MSc/Ch2-Meta-analysis/Output/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34A75613-1494-D644-BFB1-AD7F2C0E0FCA}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E53B579-787C-2E41-9EC5-361EAB8E9158}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8780" yWindow="460" windowWidth="23540" windowHeight="15840" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
+    <workbookView xWindow="3060" yWindow="460" windowWidth="23540" windowHeight="15840" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
   </bookViews>
   <sheets>
     <sheet name="Include" sheetId="1" r:id="rId1"/>
@@ -13502,7 +13502,7 @@
         <v>314</v>
       </c>
       <c r="AJ60" s="1" t="s">
-        <v>805</v>
+        <v>718</v>
       </c>
       <c r="AK60" s="1" t="s">
         <v>360</v>
@@ -13651,7 +13651,7 @@
         <v>314</v>
       </c>
       <c r="AJ61" s="1" t="s">
-        <v>718</v>
+        <v>805</v>
       </c>
       <c r="AK61" s="1" t="s">
         <v>360</v>
@@ -13800,7 +13800,7 @@
         <v>314</v>
       </c>
       <c r="AJ62" s="1" t="s">
-        <v>718</v>
+        <v>805</v>
       </c>
       <c r="AK62" s="1" t="s">
         <v>360</v>
@@ -13949,7 +13949,7 @@
         <v>314</v>
       </c>
       <c r="AJ63" s="1" t="s">
-        <v>718</v>
+        <v>805</v>
       </c>
       <c r="AK63" s="1" t="s">
         <v>360</v>
@@ -14098,7 +14098,7 @@
         <v>314</v>
       </c>
       <c r="AJ64" s="1" t="s">
-        <v>718</v>
+        <v>805</v>
       </c>
       <c r="AK64" s="1" t="s">
         <v>360</v>
@@ -14247,7 +14247,7 @@
         <v>314</v>
       </c>
       <c r="AJ65" s="1" t="s">
-        <v>718</v>
+        <v>805</v>
       </c>
       <c r="AK65" s="1" t="s">
         <v>360</v>

</xml_diff>

<commit_message>
making sure sheets match
</commit_message>
<xml_diff>
--- a/Output/Data/meta_analysis_data.xlsx
+++ b/Output/Data/meta_analysis_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11013"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilylim/Documents/MSc/Ch2-Meta-analysis/Output/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emlim/Documents/MSc/Ch2-Meta-analysis/Output/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E53B579-787C-2E41-9EC5-361EAB8E9158}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B9D777A-A66C-1D4D-811A-89F35DF3626A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3060" yWindow="460" windowWidth="23540" windowHeight="15840" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
+    <workbookView xWindow="41800" yWindow="960" windowWidth="23540" windowHeight="15840" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
   </bookViews>
   <sheets>
     <sheet name="Include" sheetId="1" r:id="rId1"/>
@@ -37115,7 +37115,7 @@
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AV34">
+  <sortState ref="A2:AV34">
     <sortCondition ref="A1"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -38420,7 +38420,7 @@
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:AX40">
+  <sortState ref="A1:AX40">
     <sortCondition ref="A1"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fixed decimal error in treatment_mean column
</commit_message>
<xml_diff>
--- a/Output/Data/meta_analysis_data.xlsx
+++ b/Output/Data/meta_analysis_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emlim/Documents/MSc/Ch2-Meta-analysis/Output/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD260D8B-CF07-9D48-80A2-D4836210D8E6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77699900-491D-6242-8B77-0FE6151AE526}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41120" yWindow="460" windowWidth="24360" windowHeight="18320" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
+    <workbookView xWindow="36200" yWindow="460" windowWidth="24360" windowHeight="18320" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
   </bookViews>
   <sheets>
     <sheet name="Include" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11394" uniqueCount="1342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11405" uniqueCount="1341">
   <si>
     <t>paper_num</t>
   </si>
@@ -4210,9 +4210,6 @@
   </si>
   <si>
     <t>shoot size</t>
-  </si>
-  <si>
-    <t>144.7.3</t>
   </si>
   <si>
     <t>measured NPP over the day, have NPP estimates for each time period. I summed the total NPP over the day and got the adjusted se by sqrt(sum of squares). The oysters are "stocked" but the seagrass is unmanipulated. Water column ammonium, nitrate, and porewater ammonium</t>
@@ -5459,7 +5456,7 @@
         <v>11.3</v>
       </c>
       <c r="BR3" s="1" t="s">
-        <v>1326</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="4" spans="1:70">
@@ -7367,7 +7364,7 @@
         <v>25</v>
       </c>
       <c r="BR12" s="1" t="s">
-        <v>1305</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="13" spans="1:70">
@@ -7579,7 +7576,7 @@
         <v>25</v>
       </c>
       <c r="BR13" s="1" t="s">
-        <v>1305</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="14" spans="1:70">
@@ -7791,7 +7788,7 @@
         <v>25</v>
       </c>
       <c r="BR14" s="1" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
     </row>
     <row r="15" spans="1:70">
@@ -8003,7 +8000,7 @@
         <v>23</v>
       </c>
       <c r="BR15" s="1" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
     </row>
     <row r="16" spans="1:70">
@@ -8215,7 +8212,7 @@
         <v>23</v>
       </c>
       <c r="BR16" s="1" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="17" spans="1:70">
@@ -8851,7 +8848,7 @@
         <v>18</v>
       </c>
       <c r="BR19" s="11" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="20" spans="1:70">
@@ -8961,7 +8958,7 @@
         <v>665</v>
       </c>
       <c r="AJ20" s="1" t="s">
-        <v>666</v>
+        <v>985</v>
       </c>
       <c r="AK20" s="1" t="s">
         <v>360</v>
@@ -9063,7 +9060,7 @@
         <v>18</v>
       </c>
       <c r="BR20" s="11" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
     </row>
     <row r="21" spans="1:70">
@@ -9173,7 +9170,7 @@
         <v>665</v>
       </c>
       <c r="AJ21" s="1" t="s">
-        <v>666</v>
+        <v>985</v>
       </c>
       <c r="AK21" s="1" t="s">
         <v>360</v>
@@ -9275,7 +9272,7 @@
         <v>18</v>
       </c>
       <c r="BR21" s="11" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
     </row>
     <row r="22" spans="1:70">
@@ -9385,7 +9382,7 @@
         <v>665</v>
       </c>
       <c r="AJ22" s="1" t="s">
-        <v>666</v>
+        <v>985</v>
       </c>
       <c r="AK22" s="1" t="s">
         <v>360</v>
@@ -9487,7 +9484,7 @@
         <v>18</v>
       </c>
       <c r="BR22" s="11" t="s">
-        <v>1304</v>
+        <v>1303</v>
       </c>
     </row>
     <row r="23" spans="1:70">
@@ -9597,7 +9594,7 @@
         <v>665</v>
       </c>
       <c r="AJ23" s="1" t="s">
-        <v>666</v>
+        <v>985</v>
       </c>
       <c r="AK23" s="1" t="s">
         <v>360</v>
@@ -9611,8 +9608,11 @@
       <c r="AN23" s="1" t="s">
         <v>314</v>
       </c>
-      <c r="AO23" s="1" t="s">
-        <v>1300</v>
+      <c r="AO23" s="1">
+        <v>144.69999999999999</v>
+      </c>
+      <c r="AP23" s="1">
+        <v>7.3</v>
       </c>
       <c r="AQ23" s="11" t="s">
         <v>314</v>
@@ -9696,7 +9696,7 @@
         <v>18</v>
       </c>
       <c r="BR23" s="11" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
     </row>
     <row r="24" spans="1:70">
@@ -9908,7 +9908,7 @@
         <v>25</v>
       </c>
       <c r="BR24" s="1" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
     </row>
     <row r="25" spans="1:70">
@@ -10120,7 +10120,7 @@
         <v>25</v>
       </c>
       <c r="BR25" s="1" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
     </row>
     <row r="26" spans="1:70">
@@ -10332,7 +10332,7 @@
         <v>25</v>
       </c>
       <c r="BR26" s="1" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
     </row>
     <row r="27" spans="1:70">
@@ -10544,7 +10544,7 @@
         <v>19.458930899999999</v>
       </c>
       <c r="BR27" s="1" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="28" spans="1:70">
@@ -10756,7 +10756,7 @@
         <v>25.725274725274684</v>
       </c>
       <c r="BR28" s="1" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
     </row>
     <row r="29" spans="1:70">
@@ -12452,7 +12452,7 @@
         <v>27.2</v>
       </c>
       <c r="BR36" s="1" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="37" spans="1:70">
@@ -12664,7 +12664,7 @@
         <v>26</v>
       </c>
       <c r="BR37" s="1" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
     </row>
     <row r="38" spans="1:70">
@@ -12876,7 +12876,7 @@
         <v>26</v>
       </c>
       <c r="BR38" s="1" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="39" spans="1:70">
@@ -13088,7 +13088,7 @@
         <v>26</v>
       </c>
       <c r="BR39" s="1" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="40" spans="1:70">
@@ -13300,7 +13300,7 @@
         <v>26</v>
       </c>
       <c r="BR40" s="1" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="41" spans="1:70">
@@ -13512,7 +13512,7 @@
         <v>26</v>
       </c>
       <c r="BR41" s="1" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="42" spans="1:70">
@@ -13724,7 +13724,7 @@
         <v>26</v>
       </c>
       <c r="BR42" s="1" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="43" spans="1:70">
@@ -13936,7 +13936,7 @@
         <v>28.65</v>
       </c>
       <c r="BR43" s="1" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="44" spans="1:70">
@@ -14148,7 +14148,7 @@
         <v>17</v>
       </c>
       <c r="BR44" s="1" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="45" spans="1:70">
@@ -14360,7 +14360,7 @@
         <v>27.94</v>
       </c>
       <c r="BR45" s="1" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="46" spans="1:70">
@@ -14572,7 +14572,7 @@
         <v>25</v>
       </c>
       <c r="BR46" s="1" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="47" spans="1:70">
@@ -14784,7 +14784,7 @@
         <v>26.17</v>
       </c>
       <c r="BR47" s="1" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="48" spans="1:70">
@@ -18388,7 +18388,7 @@
         <v>27</v>
       </c>
       <c r="BR64" s="1" t="s">
-        <v>1324</v>
+        <v>1323</v>
       </c>
     </row>
     <row r="65" spans="1:70">
@@ -27716,7 +27716,7 @@
         <v>25</v>
       </c>
       <c r="BR108" s="1" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="109" spans="1:70">
@@ -35842,6 +35842,9 @@
       <c r="V147" s="1" t="s">
         <v>602</v>
       </c>
+      <c r="W147" s="1" t="s">
+        <v>314</v>
+      </c>
       <c r="X147" s="1" t="s">
         <v>295</v>
       </c>
@@ -36051,6 +36054,9 @@
       <c r="V148" s="1" t="s">
         <v>602</v>
       </c>
+      <c r="W148" s="1" t="s">
+        <v>314</v>
+      </c>
       <c r="X148" s="1" t="s">
         <v>295</v>
       </c>
@@ -36260,6 +36266,9 @@
       <c r="V149" s="1" t="s">
         <v>602</v>
       </c>
+      <c r="W149" s="1" t="s">
+        <v>314</v>
+      </c>
       <c r="X149" s="1" t="s">
         <v>295</v>
       </c>
@@ -36469,6 +36478,9 @@
       <c r="V150" s="1" t="s">
         <v>602</v>
       </c>
+      <c r="W150" s="1" t="s">
+        <v>314</v>
+      </c>
       <c r="X150" s="1" t="s">
         <v>295</v>
       </c>
@@ -36678,6 +36690,9 @@
       <c r="V151" s="1" t="s">
         <v>602</v>
       </c>
+      <c r="W151" s="1" t="s">
+        <v>314</v>
+      </c>
       <c r="X151" s="1" t="s">
         <v>295</v>
       </c>
@@ -36887,6 +36902,9 @@
       <c r="V152" s="1" t="s">
         <v>602</v>
       </c>
+      <c r="W152" s="1" t="s">
+        <v>314</v>
+      </c>
       <c r="X152" s="1" t="s">
         <v>295</v>
       </c>
@@ -37096,6 +37114,9 @@
       <c r="V153" s="1" t="s">
         <v>574</v>
       </c>
+      <c r="W153" s="1" t="s">
+        <v>314</v>
+      </c>
       <c r="X153" s="1" t="s">
         <v>295</v>
       </c>
@@ -37305,6 +37326,9 @@
       <c r="V154" s="1" t="s">
         <v>574</v>
       </c>
+      <c r="W154" s="1" t="s">
+        <v>314</v>
+      </c>
       <c r="X154" s="1" t="s">
         <v>295</v>
       </c>
@@ -37514,6 +37538,9 @@
       <c r="V155" s="1" t="s">
         <v>574</v>
       </c>
+      <c r="W155" s="1" t="s">
+        <v>314</v>
+      </c>
       <c r="X155" s="1" t="s">
         <v>295</v>
       </c>
@@ -37723,6 +37750,9 @@
       <c r="V156" s="1" t="s">
         <v>574</v>
       </c>
+      <c r="W156" s="1" t="s">
+        <v>314</v>
+      </c>
       <c r="X156" s="1" t="s">
         <v>295</v>
       </c>
@@ -37932,6 +37962,9 @@
       <c r="V157" s="1" t="s">
         <v>574</v>
       </c>
+      <c r="W157" s="1" t="s">
+        <v>314</v>
+      </c>
       <c r="X157" s="1" t="s">
         <v>295</v>
       </c>
@@ -38141,6 +38174,9 @@
       <c r="V158" s="1" t="s">
         <v>574</v>
       </c>
+      <c r="W158" s="1" t="s">
+        <v>314</v>
+      </c>
       <c r="X158" s="1" t="s">
         <v>295</v>
       </c>
@@ -41740,7 +41776,7 @@
         <v>314</v>
       </c>
       <c r="W175" s="1" t="s">
-        <v>1327</v>
+        <v>1326</v>
       </c>
       <c r="X175" s="11" t="s">
         <v>312</v>
@@ -41788,7 +41824,7 @@
         <v>1134</v>
       </c>
       <c r="AM175" s="11" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
       <c r="AN175" s="11" t="s">
         <v>314</v>
@@ -41881,7 +41917,7 @@
         <v>26.499666666666666</v>
       </c>
       <c r="BR175" s="1" t="s">
-        <v>1341</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="176" spans="1:70">
@@ -41952,7 +41988,7 @@
         <v>314</v>
       </c>
       <c r="W176" s="1" t="s">
-        <v>1327</v>
+        <v>1326</v>
       </c>
       <c r="X176" s="11" t="s">
         <v>312</v>
@@ -42093,7 +42129,7 @@
         <v>26.499666666666666</v>
       </c>
       <c r="BR176" s="1" t="s">
-        <v>1340</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="177" spans="1:70">
@@ -42164,7 +42200,7 @@
         <v>314</v>
       </c>
       <c r="W177" s="1" t="s">
-        <v>1327</v>
+        <v>1326</v>
       </c>
       <c r="X177" s="11" t="s">
         <v>312</v>
@@ -42212,7 +42248,7 @@
         <v>1134</v>
       </c>
       <c r="AM177" s="11" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
       <c r="AN177" s="11" t="s">
         <v>314</v>
@@ -42305,7 +42341,7 @@
         <v>26.499666666666666</v>
       </c>
       <c r="BR177" s="1" t="s">
-        <v>1340</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="178" spans="1:70">
@@ -42373,7 +42409,7 @@
         <v>1</v>
       </c>
       <c r="V178" s="1" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="W178" s="1">
         <v>1981</v>
@@ -42517,7 +42553,7 @@
         <v>26.499666666666666</v>
       </c>
       <c r="BR178" s="1" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="179" spans="1:70">
@@ -42585,7 +42621,7 @@
         <v>1</v>
       </c>
       <c r="V179" s="1" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="W179" s="1">
         <v>1981</v>
@@ -42636,7 +42672,7 @@
         <v>1134</v>
       </c>
       <c r="AM179" s="11" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
       <c r="AN179" s="11" t="s">
         <v>658</v>
@@ -42729,7 +42765,7 @@
         <v>26.499666666666666</v>
       </c>
       <c r="BR179" s="1" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="180" spans="1:70">
@@ -42797,7 +42833,7 @@
         <v>1</v>
       </c>
       <c r="V180" s="1" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="W180" s="1">
         <v>1981</v>
@@ -42848,7 +42884,7 @@
         <v>1134</v>
       </c>
       <c r="AM180" s="11" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="AN180" s="11" t="s">
         <v>658</v>
@@ -42941,7 +42977,7 @@
         <v>26.499666666666666</v>
       </c>
       <c r="BR180" s="1" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="181" spans="1:70">
@@ -43009,7 +43045,7 @@
         <v>1</v>
       </c>
       <c r="V181" s="1" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="W181" s="1">
         <v>1981</v>
@@ -43060,7 +43096,7 @@
         <v>1134</v>
       </c>
       <c r="AM181" s="11" t="s">
-        <v>1331</v>
+        <v>1330</v>
       </c>
       <c r="AN181" s="11" t="s">
         <v>658</v>
@@ -43153,7 +43189,7 @@
         <v>26.499666666666666</v>
       </c>
       <c r="BR181" s="1" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="182" spans="1:70">
@@ -43221,7 +43257,7 @@
         <v>1</v>
       </c>
       <c r="V182" s="1" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="W182" s="1">
         <v>1981</v>
@@ -43365,7 +43401,7 @@
         <v>26.499666666666666</v>
       </c>
       <c r="BR182" s="1" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="183" spans="1:70">
@@ -43433,7 +43469,7 @@
         <v>1</v>
       </c>
       <c r="V183" s="1" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="W183" s="1">
         <v>1981</v>
@@ -43484,7 +43520,7 @@
         <v>1134</v>
       </c>
       <c r="AM183" s="11" t="s">
-        <v>1332</v>
+        <v>1331</v>
       </c>
       <c r="AN183" s="11" t="s">
         <v>658</v>
@@ -43577,7 +43613,7 @@
         <v>26.499666666666666</v>
       </c>
       <c r="BR183" s="1" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="184" spans="1:70">

</xml_diff>

<commit_message>
tbh im not sure what changed
</commit_message>
<xml_diff>
--- a/Output/Data/meta_analysis_data.xlsx
+++ b/Output/Data/meta_analysis_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emlim/Documents/MSc/Ch2-Meta-analysis/Output/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77699900-491D-6242-8B77-0FE6151AE526}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{332DD5A0-2595-EB40-8170-C1A37CB01AA4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="36200" yWindow="460" windowWidth="24360" windowHeight="18320" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
+    <workbookView xWindow="31920" yWindow="460" windowWidth="30920" windowHeight="19400" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
   </bookViews>
   <sheets>
     <sheet name="Include" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Changed response for peterson paper
</commit_message>
<xml_diff>
--- a/Output/Data/meta_analysis_data.xlsx
+++ b/Output/Data/meta_analysis_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emlim/Documents/MSc/Ch2-Meta-analysis/Output/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emlim/Documents/PhD/Ch1-Meta-analysis/Output/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFE7F0A8-014D-D34A-8F0F-B5710DC0B5CA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5950907-3CB6-0A43-BA09-B3A6AFF54273}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30480" yWindow="460" windowWidth="34880" windowHeight="21840" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
+    <workbookView xWindow="1600" yWindow="460" windowWidth="24520" windowHeight="15940" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
   </bookViews>
   <sheets>
     <sheet name="Include" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11669" uniqueCount="1350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11669" uniqueCount="1347">
   <si>
     <t>paper_num</t>
   </si>
@@ -4233,9 +4233,6 @@
     <t>means are mean values over the course of the experiment? It’s a 2 way fully factorial ANOVA, farm site and ref site each had + mussel pee and - mussel pee. Our treatment is the farm site + pee and the control is ref site - pee. Nh4 measured in water n = 6, nitrate and nitrite presented together n = 15. temp from (same lagoon, also oysters, just averaged august temps from both available years) https://www.mdpi.com/2077-1312/8/6/382/htm</t>
   </si>
   <si>
-    <t>Change in leaf # per shoot. This is just the 0 mussel vs 1500 mussels per m2. We're ignoring the intermediate mussel treatment. Reports max nitrate at 3, but 1.4 = avg from  https://aslopubs.onlinelibrary.wiley.com/doi/epdf/10.4319/lo.2000.45.5.1041       Temperature from https://www.int-res.com/articles/meps2020/639/m639p037.pdf</t>
-  </si>
-  <si>
     <t>high vs low grunt density. The ammonium is the predicted nh4 excretion rate in mg/m^2/day. background 1.4 = avg from  https://aslopubs.onlinelibrary.wiley.com/doi/epdf/10.4319/lo.2000.45.5.1041.     temp from https://downloads.hindawi.com/journals/jmb/2011/981723.pdf</t>
   </si>
   <si>
@@ -4281,18 +4278,6 @@
     <t>tissue dry weight</t>
   </si>
   <si>
-    <t>growth (linear extension)</t>
-  </si>
-  <si>
-    <t>surface area</t>
-  </si>
-  <si>
-    <t>volume</t>
-  </si>
-  <si>
-    <t>dry weight</t>
-  </si>
-  <si>
     <t>all year</t>
   </si>
   <si>
@@ -4305,9 +4290,6 @@
     <t xml:space="preserve">volume (cm3 per 4 months). Growth over a year. Some coral with grunts, some without. </t>
   </si>
   <si>
-    <t xml:space="preserve">density (g/cm3). Growth over a year. Some coral with grunts, some without. </t>
-  </si>
-  <si>
     <t xml:space="preserve">tissue dry weight (mg per 4 months). Growth over a year. Some coral with grunts, some without. </t>
   </si>
   <si>
@@ -4360,6 +4342,15 @@
   </si>
   <si>
     <t>mg/L/h</t>
+  </si>
+  <si>
+    <t>skeletal density</t>
+  </si>
+  <si>
+    <t xml:space="preserve">skeletal density (g/cm3). Growth over a year. Some coral with grunts, some without. </t>
+  </si>
+  <si>
+    <t>Change in leaf # per shoot. Measurement in Sept - measurement in May. This is just the 0 mussel vs 1500 mussels per m2. We're ignoring the intermediate mussel treatment. Reports max nitrate at 3, but 1.4 = avg from  https://aslopubs.onlinelibrary.wiley.com/doi/epdf/10.4319/lo.2000.45.5.1041       Temperature from https://www.int-res.com/articles/meps2020/639/m639p037.pdf</t>
   </si>
 </sst>
 </file>
@@ -4448,7 +4439,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4479,6 +4470,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -4493,7 +4490,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -4522,6 +4519,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -4840,7 +4838,9 @@
   <dimension ref="A1:BS189"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="62" width="10.83203125" style="1"/>
+    <col min="1" max="38" width="10.83203125" style="1"/>
+    <col min="39" max="39" width="10.83203125" style="22"/>
+    <col min="40" max="62" width="10.83203125" style="1"/>
     <col min="63" max="63" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="64" max="64" width="10.83203125" style="1"/>
     <col min="65" max="65" width="10.83203125" style="1" customWidth="1"/>
@@ -4965,7 +4965,7 @@
       <c r="AL1" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AM1" s="22" t="s">
         <v>316</v>
       </c>
       <c r="AN1" s="1" t="s">
@@ -5053,7 +5053,7 @@
         <v>1205</v>
       </c>
       <c r="BP1" s="1" t="s">
-        <v>1339</v>
+        <v>1333</v>
       </c>
       <c r="BQ1" s="1" t="s">
         <v>1210</v>
@@ -5180,7 +5180,7 @@
       <c r="AL2" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM2" s="1" t="s">
+      <c r="AM2" s="22" t="s">
         <v>643</v>
       </c>
       <c r="AN2" s="1" t="s">
@@ -5268,7 +5268,7 @@
         <v>1206</v>
       </c>
       <c r="BP2" s="1" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ2" s="1">
         <v>1.0649999999999999</v>
@@ -5395,7 +5395,7 @@
       <c r="AL3" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM3" s="1" t="s">
+      <c r="AM3" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN3" s="11" t="s">
@@ -5492,7 +5492,7 @@
         <v>11.3</v>
       </c>
       <c r="BS3" s="1" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="4" spans="1:71">
@@ -5610,7 +5610,7 @@
       <c r="AL4" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM4" s="1" t="s">
+      <c r="AM4" s="22" t="s">
         <v>348</v>
       </c>
       <c r="AN4" s="11" t="s">
@@ -5825,7 +5825,7 @@
       <c r="AL5" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM5" s="1" t="s">
+      <c r="AM5" s="22" t="s">
         <v>580</v>
       </c>
       <c r="AN5" s="11" t="s">
@@ -6040,7 +6040,7 @@
       <c r="AL6" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM6" s="1" t="s">
+      <c r="AM6" s="22" t="s">
         <v>866</v>
       </c>
       <c r="AN6" s="11" t="s">
@@ -6255,7 +6255,7 @@
       <c r="AL7" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM7" s="1" t="s">
+      <c r="AM7" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN7" s="11" t="s">
@@ -6470,7 +6470,7 @@
       <c r="AL8" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM8" s="11" t="s">
+      <c r="AM8" s="22" t="s">
         <v>348</v>
       </c>
       <c r="AN8" s="11" t="s">
@@ -6685,7 +6685,7 @@
       <c r="AL9" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM9" s="11" t="s">
+      <c r="AM9" s="22" t="s">
         <v>580</v>
       </c>
       <c r="AN9" s="11" t="s">
@@ -6900,7 +6900,7 @@
       <c r="AL10" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM10" s="11" t="s">
+      <c r="AM10" s="22" t="s">
         <v>866</v>
       </c>
       <c r="AN10" s="11" t="s">
@@ -7115,7 +7115,7 @@
       <c r="AL11" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM11" s="11" t="s">
+      <c r="AM11" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN11" s="11" t="s">
@@ -7330,7 +7330,7 @@
       <c r="AL12" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM12" s="11" t="s">
+      <c r="AM12" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN12" s="11" t="s">
@@ -7418,7 +7418,7 @@
         <v>1207</v>
       </c>
       <c r="BP12" s="11" t="s">
-        <v>1340</v>
+        <v>1334</v>
       </c>
       <c r="BQ12" s="11">
         <v>2.13</v>
@@ -7545,7 +7545,7 @@
       <c r="AL13" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM13" s="11" t="s">
+      <c r="AM13" s="22" t="s">
         <v>598</v>
       </c>
       <c r="AN13" s="11" t="s">
@@ -7633,7 +7633,7 @@
         <v>1207</v>
       </c>
       <c r="BP13" s="11" t="s">
-        <v>1340</v>
+        <v>1334</v>
       </c>
       <c r="BQ13" s="11">
         <v>2.13</v>
@@ -7760,7 +7760,7 @@
       <c r="AL14" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM14" s="11" t="s">
+      <c r="AM14" s="22" t="s">
         <v>348</v>
       </c>
       <c r="AN14" s="11" t="s">
@@ -7848,7 +7848,7 @@
         <v>1207</v>
       </c>
       <c r="BP14" s="11" t="s">
-        <v>1340</v>
+        <v>1334</v>
       </c>
       <c r="BQ14" s="11">
         <v>2.13</v>
@@ -7975,7 +7975,7 @@
       <c r="AL15" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM15" s="1" t="s">
+      <c r="AM15" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN15" s="1" t="s">
@@ -8063,7 +8063,7 @@
         <v>1206</v>
       </c>
       <c r="BP15" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ15" s="11">
         <v>2.7777777777777701</v>
@@ -8190,7 +8190,7 @@
       <c r="AL16" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM16" s="1" t="s">
+      <c r="AM16" s="22" t="s">
         <v>725</v>
       </c>
       <c r="AN16" s="1" t="s">
@@ -8278,7 +8278,7 @@
         <v>1206</v>
       </c>
       <c r="BP16" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ16" s="11">
         <v>2.7777777777777701</v>
@@ -8405,7 +8405,7 @@
       <c r="AL17" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM17" s="1" t="s">
+      <c r="AM17" s="22" t="s">
         <v>580</v>
       </c>
       <c r="AN17" s="1" t="s">
@@ -8493,7 +8493,7 @@
         <v>1206</v>
       </c>
       <c r="BP17" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ17">
         <v>10.616666666666667</v>
@@ -8620,7 +8620,7 @@
       <c r="AL18" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM18" s="1" t="s">
+      <c r="AM18" s="22" t="s">
         <v>580</v>
       </c>
       <c r="AN18" s="1" t="s">
@@ -8708,7 +8708,7 @@
         <v>1206</v>
       </c>
       <c r="BP18" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ18">
         <v>10.616666666666667</v>
@@ -8835,7 +8835,7 @@
       <c r="AL19" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM19" s="1" t="s">
+      <c r="AM19" s="22" t="s">
         <v>667</v>
       </c>
       <c r="AN19" s="1" t="s">
@@ -8923,7 +8923,7 @@
         <v>1206</v>
       </c>
       <c r="BP19" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ19" s="11">
         <v>1.0699999999999998</v>
@@ -9050,7 +9050,7 @@
       <c r="AL20" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM20" s="1" t="s">
+      <c r="AM20" s="22" t="s">
         <v>1296</v>
       </c>
       <c r="AN20" s="1" t="s">
@@ -9138,7 +9138,7 @@
         <v>1206</v>
       </c>
       <c r="BP20" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ20" s="11">
         <v>1.0699999999999998</v>
@@ -9265,7 +9265,7 @@
       <c r="AL21" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM21" s="1" t="s">
+      <c r="AM21" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN21" s="1" t="s">
@@ -9353,7 +9353,7 @@
         <v>1206</v>
       </c>
       <c r="BP21" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ21" s="11">
         <v>1.0699999999999998</v>
@@ -9480,7 +9480,7 @@
       <c r="AL22" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM22" s="1" t="s">
+      <c r="AM22" s="22" t="s">
         <v>348</v>
       </c>
       <c r="AN22" s="1" t="s">
@@ -9568,7 +9568,7 @@
         <v>1206</v>
       </c>
       <c r="BP22" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ22" s="11">
         <v>1.0699999999999998</v>
@@ -9695,7 +9695,7 @@
       <c r="AL23" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM23" s="1" t="s">
+      <c r="AM23" s="22" t="s">
         <v>725</v>
       </c>
       <c r="AN23" s="1" t="s">
@@ -9783,7 +9783,7 @@
         <v>1206</v>
       </c>
       <c r="BP23" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ23" s="11">
         <v>1.0699999999999998</v>
@@ -9910,7 +9910,7 @@
       <c r="AL24" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM24" s="1" t="s">
+      <c r="AM24" s="22" t="s">
         <v>596</v>
       </c>
       <c r="AN24" s="1" t="s">
@@ -10125,7 +10125,7 @@
       <c r="AL25" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM25" s="1" t="s">
+      <c r="AM25" s="22" t="s">
         <v>597</v>
       </c>
       <c r="AN25" s="1" t="s">
@@ -10340,7 +10340,7 @@
       <c r="AL26" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM26" s="1" t="s">
+      <c r="AM26" s="22" t="s">
         <v>598</v>
       </c>
       <c r="AN26" s="1" t="s">
@@ -10555,7 +10555,7 @@
       <c r="AL27" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM27" s="11" t="s">
+      <c r="AM27" s="22" t="s">
         <v>580</v>
       </c>
       <c r="AN27" s="11" t="s">
@@ -10643,7 +10643,7 @@
         <v>1206</v>
       </c>
       <c r="BP27" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ27" s="11">
         <v>3</v>
@@ -10770,7 +10770,7 @@
       <c r="AL28" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM28" s="1" t="s">
+      <c r="AM28" s="22" t="s">
         <v>589</v>
       </c>
       <c r="AN28" s="1" t="s">
@@ -10858,7 +10858,7 @@
         <v>1207</v>
       </c>
       <c r="BP28" s="11" t="s">
-        <v>1341</v>
+        <v>1335</v>
       </c>
       <c r="BQ28" s="11">
         <v>1.4</v>
@@ -10867,7 +10867,7 @@
         <v>25.725274725274684</v>
       </c>
       <c r="BS28" s="1" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
     </row>
     <row r="29" spans="1:71">
@@ -10985,7 +10985,7 @@
       <c r="AL29" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM29" s="1" t="s">
+      <c r="AM29" s="22" t="s">
         <v>1136</v>
       </c>
       <c r="AN29" s="1" t="s">
@@ -11073,7 +11073,7 @@
         <v>1207</v>
       </c>
       <c r="BP29" s="11" t="s">
-        <v>1341</v>
+        <v>1335</v>
       </c>
       <c r="BQ29" s="11">
         <v>1.4</v>
@@ -11200,7 +11200,7 @@
       <c r="AL30" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM30" s="1" t="s">
+      <c r="AM30" s="22" t="s">
         <v>1136</v>
       </c>
       <c r="AN30" s="1" t="s">
@@ -11288,7 +11288,7 @@
         <v>1207</v>
       </c>
       <c r="BP30" s="11" t="s">
-        <v>1341</v>
+        <v>1335</v>
       </c>
       <c r="BQ30" s="11">
         <v>1.4</v>
@@ -11415,7 +11415,7 @@
       <c r="AL31" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM31" s="1" t="s">
+      <c r="AM31" s="22" t="s">
         <v>1136</v>
       </c>
       <c r="AN31" s="1" t="s">
@@ -11503,7 +11503,7 @@
         <v>1207</v>
       </c>
       <c r="BP31" s="11" t="s">
-        <v>1341</v>
+        <v>1335</v>
       </c>
       <c r="BQ31" s="11">
         <v>1.4</v>
@@ -11630,7 +11630,7 @@
       <c r="AL32" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM32" s="1" t="s">
+      <c r="AM32" s="22" t="s">
         <v>1136</v>
       </c>
       <c r="AN32" s="1" t="s">
@@ -11718,7 +11718,7 @@
         <v>1207</v>
       </c>
       <c r="BP32" s="11" t="s">
-        <v>1341</v>
+        <v>1335</v>
       </c>
       <c r="BQ32" s="11">
         <v>1.4</v>
@@ -11845,7 +11845,7 @@
       <c r="AL33" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM33" s="1" t="s">
+      <c r="AM33" s="22" t="s">
         <v>1136</v>
       </c>
       <c r="AN33" s="1" t="s">
@@ -11933,7 +11933,7 @@
         <v>1207</v>
       </c>
       <c r="BP33" s="11" t="s">
-        <v>1341</v>
+        <v>1335</v>
       </c>
       <c r="BQ33" s="11">
         <v>1.4</v>
@@ -12060,7 +12060,7 @@
       <c r="AL34" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM34" s="1" t="s">
+      <c r="AM34" s="22" t="s">
         <v>1136</v>
       </c>
       <c r="AN34" s="1" t="s">
@@ -12148,7 +12148,7 @@
         <v>1207</v>
       </c>
       <c r="BP34" s="11" t="s">
-        <v>1341</v>
+        <v>1335</v>
       </c>
       <c r="BQ34" s="11">
         <v>1.4</v>
@@ -12275,7 +12275,7 @@
       <c r="AL35" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM35" s="1" t="s">
+      <c r="AM35" s="22" t="s">
         <v>1136</v>
       </c>
       <c r="AN35" s="1" t="s">
@@ -12363,7 +12363,7 @@
         <v>1207</v>
       </c>
       <c r="BP35" s="11" t="s">
-        <v>1341</v>
+        <v>1335</v>
       </c>
       <c r="BQ35" s="11">
         <v>1.4</v>
@@ -12490,7 +12490,7 @@
       <c r="AL36" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM36" s="1" t="s">
+      <c r="AM36" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN36" s="1" t="s">
@@ -12578,7 +12578,7 @@
         <v>819</v>
       </c>
       <c r="BP36" s="11" t="s">
-        <v>1349</v>
+        <v>1343</v>
       </c>
       <c r="BQ36" s="11">
         <v>2.13</v>
@@ -12587,7 +12587,7 @@
         <v>27.2</v>
       </c>
       <c r="BS36" s="1" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="37" spans="1:71">
@@ -12705,7 +12705,7 @@
       <c r="AL37" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM37" s="1" t="s">
+      <c r="AM37" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN37" s="1" t="s">
@@ -12793,7 +12793,7 @@
         <v>1206</v>
       </c>
       <c r="BP37" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ37">
         <v>6.3507812955294964</v>
@@ -12802,7 +12802,7 @@
         <v>26</v>
       </c>
       <c r="BS37" s="1" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="38" spans="1:71">
@@ -12920,7 +12920,7 @@
       <c r="AL38" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM38" s="1" t="s">
+      <c r="AM38" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN38" s="1" t="s">
@@ -13008,7 +13008,7 @@
         <v>1206</v>
       </c>
       <c r="BP38" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ38">
         <v>8.6337418919616322</v>
@@ -13017,7 +13017,7 @@
         <v>26</v>
       </c>
       <c r="BS38" s="1" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="39" spans="1:71">
@@ -13135,7 +13135,7 @@
       <c r="AL39" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM39" s="1" t="s">
+      <c r="AM39" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN39" s="1" t="s">
@@ -13223,7 +13223,7 @@
         <v>1206</v>
       </c>
       <c r="BP39" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ39">
         <v>7.5545241554664546</v>
@@ -13232,7 +13232,7 @@
         <v>26</v>
       </c>
       <c r="BS39" s="1" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
     </row>
     <row r="40" spans="1:71">
@@ -13350,7 +13350,7 @@
       <c r="AL40" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM40" s="1" t="s">
+      <c r="AM40" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN40" s="1" t="s">
@@ -13438,7 +13438,7 @@
         <v>1206</v>
       </c>
       <c r="BP40" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ40">
         <v>9.9620098753403727</v>
@@ -13447,7 +13447,7 @@
         <v>26</v>
       </c>
       <c r="BS40" s="1" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="41" spans="1:71">
@@ -13565,7 +13565,7 @@
       <c r="AL41" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM41" s="1" t="s">
+      <c r="AM41" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN41" s="1" t="s">
@@ -13653,7 +13653,7 @@
         <v>1206</v>
       </c>
       <c r="BP41" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ41">
         <v>7.4715074065052436</v>
@@ -13662,7 +13662,7 @@
         <v>26</v>
       </c>
       <c r="BS41" s="1" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
     </row>
     <row r="42" spans="1:71">
@@ -13780,7 +13780,7 @@
       <c r="AL42" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM42" s="1" t="s">
+      <c r="AM42" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN42" s="1" t="s">
@@ -13868,7 +13868,7 @@
         <v>1206</v>
       </c>
       <c r="BP42" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ42">
         <v>7.6375409044275955</v>
@@ -13877,7 +13877,7 @@
         <v>26</v>
       </c>
       <c r="BS42" s="1" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="43" spans="1:71">
@@ -13995,7 +13995,7 @@
       <c r="AL43" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM43" s="1" t="s">
+      <c r="AM43" s="22" t="s">
         <v>580</v>
       </c>
       <c r="AN43" s="1" t="s">
@@ -14092,7 +14092,7 @@
         <v>28.65</v>
       </c>
       <c r="BS43" s="1" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="44" spans="1:71">
@@ -14210,7 +14210,7 @@
       <c r="AL44" s="1" t="s">
         <v>819</v>
       </c>
-      <c r="AM44" s="1" t="s">
+      <c r="AM44" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN44" s="1" t="s">
@@ -14298,7 +14298,7 @@
         <v>1206</v>
       </c>
       <c r="BP44" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ44" s="11" t="s">
         <v>314</v>
@@ -14307,7 +14307,7 @@
         <v>17</v>
       </c>
       <c r="BS44" s="1" t="s">
-        <v>1344</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="45" spans="1:71">
@@ -14425,7 +14425,7 @@
       <c r="AL45" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM45" s="1" t="s">
+      <c r="AM45" s="22" t="s">
         <v>696</v>
       </c>
       <c r="AN45" s="1" t="s">
@@ -14522,7 +14522,7 @@
         <v>27.94</v>
       </c>
       <c r="BS45" s="1" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="46" spans="1:71">
@@ -14640,7 +14640,7 @@
       <c r="AL46" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM46" s="1" t="s">
+      <c r="AM46" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN46" s="1" t="s">
@@ -14728,7 +14728,7 @@
         <v>1207</v>
       </c>
       <c r="BP46" s="11" t="s">
-        <v>1340</v>
+        <v>1334</v>
       </c>
       <c r="BQ46" s="11">
         <v>2.13</v>
@@ -14737,7 +14737,7 @@
         <v>25</v>
       </c>
       <c r="BS46" s="1" t="s">
-        <v>1338</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="47" spans="1:71">
@@ -14855,7 +14855,7 @@
       <c r="AL47" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM47" s="1" t="s">
+      <c r="AM47" s="22" t="s">
         <v>1146</v>
       </c>
       <c r="AN47" s="1" t="s">
@@ -14943,7 +14943,7 @@
         <v>1206</v>
       </c>
       <c r="BP47" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ47" s="1">
         <v>0.16129032258064363</v>
@@ -14952,7 +14952,7 @@
         <v>26.17</v>
       </c>
       <c r="BS47" s="1" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="48" spans="1:71">
@@ -15070,7 +15070,7 @@
       <c r="AL48" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM48" s="1" t="s">
+      <c r="AM48" s="22" t="s">
         <v>1147</v>
       </c>
       <c r="AN48" s="1" t="s">
@@ -15158,7 +15158,7 @@
         <v>1206</v>
       </c>
       <c r="BP48" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ48" s="1">
         <v>0.16129032258064363</v>
@@ -15285,7 +15285,7 @@
       <c r="AL49" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM49" s="1" t="s">
+      <c r="AM49" s="22" t="s">
         <v>1147</v>
       </c>
       <c r="AN49" s="1" t="s">
@@ -15373,7 +15373,7 @@
         <v>1206</v>
       </c>
       <c r="BP49" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ49" s="1">
         <v>0.16129032258064363</v>
@@ -15500,7 +15500,7 @@
       <c r="AL50" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM50" s="1" t="s">
+      <c r="AM50" s="22" t="s">
         <v>1147</v>
       </c>
       <c r="AN50" s="1" t="s">
@@ -15588,7 +15588,7 @@
         <v>1206</v>
       </c>
       <c r="BP50" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ50" s="1">
         <v>0.16129032258064363</v>
@@ -15715,7 +15715,7 @@
       <c r="AL51" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM51" s="1" t="s">
+      <c r="AM51" s="22" t="s">
         <v>1148</v>
       </c>
       <c r="AN51" s="1" t="s">
@@ -15803,7 +15803,7 @@
         <v>1206</v>
       </c>
       <c r="BP51" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ51" s="1">
         <v>0.16129032258064363</v>
@@ -15930,7 +15930,7 @@
       <c r="AL52" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM52" s="1" t="s">
+      <c r="AM52" s="22" t="s">
         <v>1148</v>
       </c>
       <c r="AN52" s="1" t="s">
@@ -16018,7 +16018,7 @@
         <v>1206</v>
       </c>
       <c r="BP52" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ52" s="1">
         <v>0.16129032258064363</v>
@@ -16145,7 +16145,7 @@
       <c r="AL53" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM53" s="1" t="s">
+      <c r="AM53" s="22" t="s">
         <v>1148</v>
       </c>
       <c r="AN53" s="1" t="s">
@@ -16233,7 +16233,7 @@
         <v>1206</v>
       </c>
       <c r="BP53" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ53" s="1">
         <v>0.16129032258064363</v>
@@ -16360,7 +16360,7 @@
       <c r="AL54" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM54" s="1" t="s">
+      <c r="AM54" s="22" t="s">
         <v>1008</v>
       </c>
       <c r="AN54" s="1" t="s">
@@ -16448,7 +16448,7 @@
         <v>1206</v>
       </c>
       <c r="BP54" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ54" s="11">
         <v>0.15053763440860024</v>
@@ -16575,7 +16575,7 @@
       <c r="AL55" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM55" s="1" t="s">
+      <c r="AM55" s="22" t="s">
         <v>1008</v>
       </c>
       <c r="AN55" s="1" t="s">
@@ -16663,7 +16663,7 @@
         <v>1206</v>
       </c>
       <c r="BP55" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ55" s="11">
         <v>0.17204301075268699</v>
@@ -16790,7 +16790,7 @@
       <c r="AL56" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM56" s="1" t="s">
+      <c r="AM56" s="22" t="s">
         <v>1008</v>
       </c>
       <c r="AN56" s="1" t="s">
@@ -16878,7 +16878,7 @@
         <v>1206</v>
       </c>
       <c r="BP56" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ56" s="11">
         <v>6.5217391304347394E-2</v>
@@ -17005,7 +17005,7 @@
       <c r="AL57" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM57" s="1" t="s">
+      <c r="AM57" s="22" t="s">
         <v>1008</v>
       </c>
       <c r="AN57" s="1" t="s">
@@ -17093,7 +17093,7 @@
         <v>1206</v>
       </c>
       <c r="BP57" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ57" s="11">
         <v>0.47826086956521702</v>
@@ -17220,7 +17220,7 @@
       <c r="AL58" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM58" s="1" t="s">
+      <c r="AM58" s="22" t="s">
         <v>1008</v>
       </c>
       <c r="AN58" s="1" t="s">
@@ -17308,7 +17308,7 @@
         <v>1206</v>
       </c>
       <c r="BP58" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ58" s="11">
         <v>0.14388489208633001</v>
@@ -17435,7 +17435,7 @@
       <c r="AL59" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM59" s="1" t="s">
+      <c r="AM59" s="22" t="s">
         <v>1008</v>
       </c>
       <c r="AN59" s="1" t="s">
@@ -17523,7 +17523,7 @@
         <v>1206</v>
       </c>
       <c r="BP59" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ59" s="11">
         <v>0.15053763440860024</v>
@@ -17650,7 +17650,7 @@
       <c r="AL60" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM60" s="1" t="s">
+      <c r="AM60" s="22" t="s">
         <v>1008</v>
       </c>
       <c r="AN60" s="1" t="s">
@@ -17738,7 +17738,7 @@
         <v>1206</v>
       </c>
       <c r="BP60" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ60" s="11">
         <v>0.17204301075268699</v>
@@ -17865,7 +17865,7 @@
       <c r="AL61" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM61" s="1" t="s">
+      <c r="AM61" s="22" t="s">
         <v>1008</v>
       </c>
       <c r="AN61" s="1" t="s">
@@ -17953,7 +17953,7 @@
         <v>1206</v>
       </c>
       <c r="BP61" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ61" s="11">
         <v>6.5217391304347394E-2</v>
@@ -18080,7 +18080,7 @@
       <c r="AL62" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM62" s="1" t="s">
+      <c r="AM62" s="22" t="s">
         <v>1008</v>
       </c>
       <c r="AN62" s="1" t="s">
@@ -18168,7 +18168,7 @@
         <v>1206</v>
       </c>
       <c r="BP62" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ62" s="11">
         <v>0.47826086956521702</v>
@@ -18295,7 +18295,7 @@
       <c r="AL63" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM63" s="1" t="s">
+      <c r="AM63" s="22" t="s">
         <v>1008</v>
       </c>
       <c r="AN63" s="1" t="s">
@@ -18383,7 +18383,7 @@
         <v>1206</v>
       </c>
       <c r="BP63" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ63" s="11">
         <v>0.14388489208633001</v>
@@ -18510,7 +18510,7 @@
       <c r="AL64" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM64" s="1" t="s">
+      <c r="AM64" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN64" s="1" t="s">
@@ -18598,7 +18598,7 @@
         <v>1207</v>
       </c>
       <c r="BP64" s="1" t="s">
-        <v>1348</v>
+        <v>1342</v>
       </c>
       <c r="BQ64" s="11">
         <v>0.43</v>
@@ -18607,7 +18607,7 @@
         <v>27</v>
       </c>
       <c r="BS64" s="1" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="65" spans="1:71">
@@ -18725,7 +18725,7 @@
       <c r="AL65" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM65" s="1" t="s">
+      <c r="AM65" s="22" t="s">
         <v>580</v>
       </c>
       <c r="AN65" s="1" t="s">
@@ -18813,7 +18813,7 @@
         <v>1206</v>
       </c>
       <c r="BP65" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ65" s="11">
         <v>0.92648599819331412</v>
@@ -18940,7 +18940,7 @@
       <c r="AL66" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM66" s="1" t="s">
+      <c r="AM66" s="22" t="s">
         <v>716</v>
       </c>
       <c r="AN66" s="1" t="s">
@@ -19028,7 +19028,7 @@
         <v>1206</v>
       </c>
       <c r="BP66" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ66" s="11">
         <v>0.79214092140921299</v>
@@ -19155,7 +19155,7 @@
       <c r="AL67" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM67" s="1" t="s">
+      <c r="AM67" s="22" t="s">
         <v>716</v>
       </c>
       <c r="AN67" s="1" t="s">
@@ -19243,7 +19243,7 @@
         <v>1206</v>
       </c>
       <c r="BP67" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ67" s="11">
         <v>0.90614272809394603</v>
@@ -19370,7 +19370,7 @@
       <c r="AL68" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM68" s="1" t="s">
+      <c r="AM68" s="22" t="s">
         <v>716</v>
       </c>
       <c r="AN68" s="1" t="s">
@@ -19458,7 +19458,7 @@
         <v>1206</v>
       </c>
       <c r="BP68" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ68" s="11">
         <v>1.2923215898825648</v>
@@ -19585,7 +19585,7 @@
       <c r="AL69" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM69" s="1" t="s">
+      <c r="AM69" s="22" t="s">
         <v>716</v>
       </c>
       <c r="AN69" s="1" t="s">
@@ -19673,7 +19673,7 @@
         <v>1206</v>
       </c>
       <c r="BP69" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ69" s="11">
         <v>0.54272809394760502</v>
@@ -19800,7 +19800,7 @@
       <c r="AL70" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM70" s="1" t="s">
+      <c r="AM70" s="22" t="s">
         <v>716</v>
       </c>
       <c r="AN70" s="1" t="s">
@@ -19888,7 +19888,7 @@
         <v>1206</v>
       </c>
       <c r="BP70" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ70" s="11">
         <v>1.0990966576332419</v>
@@ -20015,7 +20015,7 @@
       <c r="AL71" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM71" s="1" t="s">
+      <c r="AM71" s="22" t="s">
         <v>1008</v>
       </c>
       <c r="AN71" s="1" t="s">
@@ -20103,7 +20103,7 @@
         <v>1206</v>
       </c>
       <c r="BP71" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ71" s="11">
         <v>14.34291139240506</v>
@@ -20230,7 +20230,7 @@
       <c r="AL72" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM72" s="1" t="s">
+      <c r="AM72" s="22" t="s">
         <v>1008</v>
       </c>
       <c r="AN72" s="1" t="s">
@@ -20318,7 +20318,7 @@
         <v>1206</v>
       </c>
       <c r="BP72" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ72" s="11">
         <v>14.34291139240506</v>
@@ -20445,7 +20445,7 @@
       <c r="AL73" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM73" s="1" t="s">
+      <c r="AM73" s="22" t="s">
         <v>1008</v>
       </c>
       <c r="AN73" s="1" t="s">
@@ -20533,7 +20533,7 @@
         <v>1206</v>
       </c>
       <c r="BP73" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ73" s="11">
         <v>14.34291139240506</v>
@@ -20660,7 +20660,7 @@
       <c r="AL74" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM74" s="1" t="s">
+      <c r="AM74" s="22" t="s">
         <v>1008</v>
       </c>
       <c r="AN74" s="1" t="s">
@@ -20748,7 +20748,7 @@
         <v>1206</v>
       </c>
       <c r="BP74" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ74" s="11">
         <v>14.34291139240506</v>
@@ -20875,7 +20875,7 @@
       <c r="AL75" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM75" s="1" t="s">
+      <c r="AM75" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN75" s="1" t="s">
@@ -20963,7 +20963,7 @@
         <v>1206</v>
       </c>
       <c r="BP75" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ75" s="11">
         <v>14.34291139240506</v>
@@ -21090,7 +21090,7 @@
       <c r="AL76" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM76" s="1" t="s">
+      <c r="AM76" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN76" s="1" t="s">
@@ -21178,7 +21178,7 @@
         <v>1206</v>
       </c>
       <c r="BP76" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ76" s="11">
         <v>14.34291139240506</v>
@@ -21305,7 +21305,7 @@
       <c r="AL77" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM77" s="1" t="s">
+      <c r="AM77" s="22" t="s">
         <v>1008</v>
       </c>
       <c r="AN77" s="1" t="s">
@@ -21393,7 +21393,7 @@
         <v>1206</v>
       </c>
       <c r="BP77" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ77" s="11">
         <v>14.34291139240506</v>
@@ -21520,7 +21520,7 @@
       <c r="AL78" s="1" t="s">
         <v>1164</v>
       </c>
-      <c r="AM78" s="1" t="s">
+      <c r="AM78" s="22" t="s">
         <v>730</v>
       </c>
       <c r="AN78" s="1" t="s">
@@ -21608,7 +21608,7 @@
         <v>1206</v>
       </c>
       <c r="BP78" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ78" s="11">
         <v>23</v>
@@ -21735,7 +21735,7 @@
       <c r="AL79" s="1" t="s">
         <v>1164</v>
       </c>
-      <c r="AM79" s="1" t="s">
+      <c r="AM79" s="22" t="s">
         <v>598</v>
       </c>
       <c r="AN79" s="1" t="s">
@@ -21823,7 +21823,7 @@
         <v>1206</v>
       </c>
       <c r="BP79" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ79" s="11">
         <v>23</v>
@@ -21950,7 +21950,7 @@
       <c r="AL80" s="1" t="s">
         <v>1164</v>
       </c>
-      <c r="AM80" s="1" t="s">
+      <c r="AM80" s="22" t="s">
         <v>725</v>
       </c>
       <c r="AN80" s="1" t="s">
@@ -22038,7 +22038,7 @@
         <v>1206</v>
       </c>
       <c r="BP80" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ80" s="11">
         <v>23</v>
@@ -22165,7 +22165,7 @@
       <c r="AL81" s="1" t="s">
         <v>819</v>
       </c>
-      <c r="AM81" s="1" t="s">
+      <c r="AM81" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN81" s="1" t="s">
@@ -22253,7 +22253,7 @@
         <v>1206</v>
       </c>
       <c r="BP81" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ81" s="11">
         <v>23</v>
@@ -22380,7 +22380,7 @@
       <c r="AL82" s="1" t="s">
         <v>819</v>
       </c>
-      <c r="AM82" s="1" t="s">
+      <c r="AM82" s="22" t="s">
         <v>730</v>
       </c>
       <c r="AN82" s="1" t="s">
@@ -22468,7 +22468,7 @@
         <v>1206</v>
       </c>
       <c r="BP82" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ82" s="11">
         <v>23</v>
@@ -22595,7 +22595,7 @@
       <c r="AL83" s="1" t="s">
         <v>819</v>
       </c>
-      <c r="AM83" s="1" t="s">
+      <c r="AM83" s="22" t="s">
         <v>731</v>
       </c>
       <c r="AN83" s="1" t="s">
@@ -22683,7 +22683,7 @@
         <v>1206</v>
       </c>
       <c r="BP83" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ83" s="11">
         <v>23</v>
@@ -22810,7 +22810,7 @@
       <c r="AL84" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM84" s="1" t="s">
+      <c r="AM84" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN84" s="1" t="s">
@@ -22898,7 +22898,7 @@
         <v>1206</v>
       </c>
       <c r="BP84" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ84" s="11">
         <v>0.43</v>
@@ -23025,7 +23025,7 @@
       <c r="AL85" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM85" s="1" t="s">
+      <c r="AM85" s="22" t="s">
         <v>731</v>
       </c>
       <c r="AN85" s="1" t="s">
@@ -23113,7 +23113,7 @@
         <v>1206</v>
       </c>
       <c r="BP85" s="11" t="s">
-        <v>1345</v>
+        <v>1339</v>
       </c>
       <c r="BQ85" s="11">
         <v>11</v>
@@ -23240,7 +23240,7 @@
       <c r="AL86" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM86" s="1" t="s">
+      <c r="AM86" s="22" t="s">
         <v>598</v>
       </c>
       <c r="AN86" s="1" t="s">
@@ -23328,7 +23328,7 @@
         <v>1206</v>
       </c>
       <c r="BP86" s="11" t="s">
-        <v>1345</v>
+        <v>1339</v>
       </c>
       <c r="BQ86" s="11">
         <v>11</v>
@@ -23455,7 +23455,7 @@
       <c r="AL87" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM87" s="1" t="s">
+      <c r="AM87" s="22" t="s">
         <v>743</v>
       </c>
       <c r="AN87" s="1" t="s">
@@ -23543,7 +23543,7 @@
         <v>1206</v>
       </c>
       <c r="BP87" s="11" t="s">
-        <v>1345</v>
+        <v>1339</v>
       </c>
       <c r="BQ87" s="11">
         <v>11</v>
@@ -23670,7 +23670,7 @@
       <c r="AL88" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM88" s="1" t="s">
+      <c r="AM88" s="22" t="s">
         <v>730</v>
       </c>
       <c r="AN88" s="1" t="s">
@@ -23758,7 +23758,7 @@
         <v>1206</v>
       </c>
       <c r="BP88" s="11" t="s">
-        <v>1345</v>
+        <v>1339</v>
       </c>
       <c r="BQ88" s="11">
         <v>11</v>
@@ -23885,7 +23885,7 @@
       <c r="AL89" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM89" s="1" t="s">
+      <c r="AM89" s="22" t="s">
         <v>725</v>
       </c>
       <c r="AN89" s="1" t="s">
@@ -23973,7 +23973,7 @@
         <v>1206</v>
       </c>
       <c r="BP89" s="11" t="s">
-        <v>1345</v>
+        <v>1339</v>
       </c>
       <c r="BQ89" s="11">
         <v>11</v>
@@ -24100,7 +24100,7 @@
       <c r="AL90" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM90" s="1" t="s">
+      <c r="AM90" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN90" s="1" t="s">
@@ -24188,7 +24188,7 @@
         <v>1206</v>
       </c>
       <c r="BP90" s="11" t="s">
-        <v>1345</v>
+        <v>1339</v>
       </c>
       <c r="BQ90" s="11">
         <v>11</v>
@@ -24315,7 +24315,7 @@
       <c r="AL91" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM91" s="1" t="s">
+      <c r="AM91" s="22" t="s">
         <v>731</v>
       </c>
       <c r="AN91" s="1" t="s">
@@ -24403,7 +24403,7 @@
         <v>1206</v>
       </c>
       <c r="BP91" s="11" t="s">
-        <v>1345</v>
+        <v>1339</v>
       </c>
       <c r="BQ91" s="11">
         <v>11</v>
@@ -24530,7 +24530,7 @@
       <c r="AL92" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM92" s="1" t="s">
+      <c r="AM92" s="22" t="s">
         <v>598</v>
       </c>
       <c r="AN92" s="1" t="s">
@@ -24618,7 +24618,7 @@
         <v>1206</v>
       </c>
       <c r="BP92" s="11" t="s">
-        <v>1345</v>
+        <v>1339</v>
       </c>
       <c r="BQ92" s="11">
         <v>11</v>
@@ -24745,7 +24745,7 @@
       <c r="AL93" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM93" s="1" t="s">
+      <c r="AM93" s="22" t="s">
         <v>743</v>
       </c>
       <c r="AN93" s="1" t="s">
@@ -24833,7 +24833,7 @@
         <v>1206</v>
       </c>
       <c r="BP93" s="11" t="s">
-        <v>1345</v>
+        <v>1339</v>
       </c>
       <c r="BQ93" s="11">
         <v>11</v>
@@ -24960,7 +24960,7 @@
       <c r="AL94" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM94" s="1" t="s">
+      <c r="AM94" s="22" t="s">
         <v>730</v>
       </c>
       <c r="AN94" s="1" t="s">
@@ -25048,7 +25048,7 @@
         <v>1206</v>
       </c>
       <c r="BP94" s="11" t="s">
-        <v>1345</v>
+        <v>1339</v>
       </c>
       <c r="BQ94" s="11">
         <v>11</v>
@@ -25175,7 +25175,7 @@
       <c r="AL95" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM95" s="1" t="s">
+      <c r="AM95" s="22" t="s">
         <v>725</v>
       </c>
       <c r="AN95" s="1" t="s">
@@ -25263,7 +25263,7 @@
         <v>1206</v>
       </c>
       <c r="BP95" s="11" t="s">
-        <v>1345</v>
+        <v>1339</v>
       </c>
       <c r="BQ95" s="11">
         <v>11</v>
@@ -25390,7 +25390,7 @@
       <c r="AL96" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM96" s="1" t="s">
+      <c r="AM96" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN96" s="1" t="s">
@@ -25478,7 +25478,7 @@
         <v>1206</v>
       </c>
       <c r="BP96" s="11" t="s">
-        <v>1345</v>
+        <v>1339</v>
       </c>
       <c r="BQ96" s="11">
         <v>11</v>
@@ -25605,7 +25605,7 @@
       <c r="AL97" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM97" s="1" t="s">
+      <c r="AM97" s="22" t="s">
         <v>731</v>
       </c>
       <c r="AN97" s="1" t="s">
@@ -25693,7 +25693,7 @@
         <v>1206</v>
       </c>
       <c r="BP97" s="11" t="s">
-        <v>1345</v>
+        <v>1339</v>
       </c>
       <c r="BQ97" s="11">
         <v>11</v>
@@ -25820,7 +25820,7 @@
       <c r="AL98" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM98" s="1" t="s">
+      <c r="AM98" s="22" t="s">
         <v>598</v>
       </c>
       <c r="AN98" s="1" t="s">
@@ -25908,7 +25908,7 @@
         <v>1206</v>
       </c>
       <c r="BP98" s="11" t="s">
-        <v>1345</v>
+        <v>1339</v>
       </c>
       <c r="BQ98" s="11">
         <v>11</v>
@@ -26035,7 +26035,7 @@
       <c r="AL99" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM99" s="1" t="s">
+      <c r="AM99" s="22" t="s">
         <v>743</v>
       </c>
       <c r="AN99" s="1" t="s">
@@ -26123,7 +26123,7 @@
         <v>1206</v>
       </c>
       <c r="BP99" s="11" t="s">
-        <v>1345</v>
+        <v>1339</v>
       </c>
       <c r="BQ99" s="11">
         <v>11</v>
@@ -26250,7 +26250,7 @@
       <c r="AL100" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM100" s="1" t="s">
+      <c r="AM100" s="22" t="s">
         <v>730</v>
       </c>
       <c r="AN100" s="1" t="s">
@@ -26338,7 +26338,7 @@
         <v>1206</v>
       </c>
       <c r="BP100" s="11" t="s">
-        <v>1345</v>
+        <v>1339</v>
       </c>
       <c r="BQ100" s="11">
         <v>11</v>
@@ -26465,7 +26465,7 @@
       <c r="AL101" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM101" s="1" t="s">
+      <c r="AM101" s="22" t="s">
         <v>725</v>
       </c>
       <c r="AN101" s="1" t="s">
@@ -26553,7 +26553,7 @@
         <v>1206</v>
       </c>
       <c r="BP101" s="11" t="s">
-        <v>1345</v>
+        <v>1339</v>
       </c>
       <c r="BQ101" s="11">
         <v>11</v>
@@ -26680,7 +26680,7 @@
       <c r="AL102" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM102" s="1" t="s">
+      <c r="AM102" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN102" s="1" t="s">
@@ -26768,7 +26768,7 @@
         <v>1206</v>
       </c>
       <c r="BP102" s="11" t="s">
-        <v>1345</v>
+        <v>1339</v>
       </c>
       <c r="BQ102" s="11">
         <v>11</v>
@@ -26895,7 +26895,7 @@
       <c r="AL103" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM103" s="1" t="s">
+      <c r="AM103" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN103" s="1" t="s">
@@ -26983,7 +26983,7 @@
         <v>1206</v>
       </c>
       <c r="BP103" s="11" t="s">
-        <v>1345</v>
+        <v>1339</v>
       </c>
       <c r="BQ103" s="11">
         <v>11</v>
@@ -27110,7 +27110,7 @@
       <c r="AL104" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM104" s="1" t="s">
+      <c r="AM104" s="22" t="s">
         <v>754</v>
       </c>
       <c r="AN104" s="1" t="s">
@@ -27198,7 +27198,7 @@
         <v>1206</v>
       </c>
       <c r="BP104" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ104" s="1">
         <v>0.1</v>
@@ -27207,7 +27207,7 @@
         <v>23</v>
       </c>
       <c r="BS104" s="1" t="s">
-        <v>1346</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="105" spans="1:71">
@@ -27325,7 +27325,7 @@
       <c r="AL105" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM105" s="1" t="s">
+      <c r="AM105" s="22" t="s">
         <v>889</v>
       </c>
       <c r="AN105" s="1" t="s">
@@ -27413,7 +27413,7 @@
         <v>1206</v>
       </c>
       <c r="BP105" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ105" s="1">
         <v>0.1</v>
@@ -27540,7 +27540,7 @@
       <c r="AL106" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM106" s="1" t="s">
+      <c r="AM106" s="22" t="s">
         <v>763</v>
       </c>
       <c r="AN106" s="1" t="s">
@@ -27628,7 +27628,7 @@
         <v>819</v>
       </c>
       <c r="BP106" s="11" t="s">
-        <v>1347</v>
+        <v>1341</v>
       </c>
       <c r="BQ106" s="11">
         <v>2.0993975903614448</v>
@@ -27755,7 +27755,7 @@
       <c r="AL107" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM107" s="11" t="s">
+      <c r="AM107" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN107" s="11" t="s">
@@ -27843,7 +27843,7 @@
         <v>1206</v>
       </c>
       <c r="BP107" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ107" s="11">
         <v>1</v>
@@ -27970,7 +27970,7 @@
       <c r="AL108" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM108" s="1" t="s">
+      <c r="AM108" s="22" t="s">
         <v>730</v>
       </c>
       <c r="AN108" s="1" t="s">
@@ -28067,7 +28067,7 @@
         <v>25</v>
       </c>
       <c r="BS108" s="1" t="s">
-        <v>1307</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="109" spans="1:71">
@@ -28185,7 +28185,7 @@
       <c r="AL109" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM109" s="1" t="s">
+      <c r="AM109" s="22" t="s">
         <v>773</v>
       </c>
       <c r="AN109" s="1" t="s">
@@ -28273,7 +28273,7 @@
         <v>1206</v>
       </c>
       <c r="BP109" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ109" s="11">
         <v>1.4</v>
@@ -28400,7 +28400,7 @@
       <c r="AL110" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM110" s="1" t="s">
+      <c r="AM110" s="22" t="s">
         <v>774</v>
       </c>
       <c r="AN110" s="1" t="s">
@@ -28488,7 +28488,7 @@
         <v>1206</v>
       </c>
       <c r="BP110" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ110" s="11">
         <v>1.4</v>
@@ -28615,8 +28615,8 @@
       <c r="AL111" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM111" s="1" t="s">
-        <v>775</v>
+      <c r="AM111" s="22" t="s">
+        <v>317</v>
       </c>
       <c r="AN111" s="1" t="s">
         <v>658</v>
@@ -28703,7 +28703,7 @@
         <v>1206</v>
       </c>
       <c r="BP111" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ111" s="11">
         <v>1.4</v>
@@ -28830,8 +28830,8 @@
       <c r="AL112" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM112" s="1" t="s">
-        <v>775</v>
+      <c r="AM112" s="22" t="s">
+        <v>317</v>
       </c>
       <c r="AN112" s="1" t="s">
         <v>658</v>
@@ -28918,7 +28918,7 @@
         <v>1206</v>
       </c>
       <c r="BP112" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ112" s="11">
         <v>1.4</v>
@@ -29045,8 +29045,8 @@
       <c r="AL113" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM113" s="1" t="s">
-        <v>775</v>
+      <c r="AM113" s="22" t="s">
+        <v>317</v>
       </c>
       <c r="AN113" s="1" t="s">
         <v>658</v>
@@ -29133,7 +29133,7 @@
         <v>1206</v>
       </c>
       <c r="BP113" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ113" s="11">
         <v>1.4</v>
@@ -29260,8 +29260,8 @@
       <c r="AL114" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM114" s="1" t="s">
-        <v>775</v>
+      <c r="AM114" s="22" t="s">
+        <v>317</v>
       </c>
       <c r="AN114" s="1" t="s">
         <v>658</v>
@@ -29348,7 +29348,7 @@
         <v>1206</v>
       </c>
       <c r="BP114" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ114" s="11">
         <v>1.4</v>
@@ -29475,8 +29475,8 @@
       <c r="AL115" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM115" s="1" t="s">
-        <v>775</v>
+      <c r="AM115" s="22" t="s">
+        <v>317</v>
       </c>
       <c r="AN115" s="1" t="s">
         <v>658</v>
@@ -29563,7 +29563,7 @@
         <v>1206</v>
       </c>
       <c r="BP115" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ115" s="11">
         <v>1.4</v>
@@ -29690,7 +29690,7 @@
       <c r="AL116" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM116" s="1" t="s">
+      <c r="AM116" s="22" t="s">
         <v>775</v>
       </c>
       <c r="AN116" s="1" t="s">
@@ -29778,7 +29778,7 @@
         <v>1206</v>
       </c>
       <c r="BP116" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ116">
         <v>1.58</v>
@@ -29905,7 +29905,7 @@
       <c r="AL117" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM117" s="1" t="s">
+      <c r="AM117" s="22" t="s">
         <v>775</v>
       </c>
       <c r="AN117" s="1" t="s">
@@ -29993,7 +29993,7 @@
         <v>1206</v>
       </c>
       <c r="BP117" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ117">
         <v>1.58</v>
@@ -30120,7 +30120,7 @@
       <c r="AL118" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM118" s="1" t="s">
+      <c r="AM118" s="22" t="s">
         <v>775</v>
       </c>
       <c r="AN118" s="1" t="s">
@@ -30208,7 +30208,7 @@
         <v>1206</v>
       </c>
       <c r="BP118" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ118">
         <v>1.58</v>
@@ -30335,7 +30335,7 @@
       <c r="AL119" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM119" s="1" t="s">
+      <c r="AM119" s="22" t="s">
         <v>775</v>
       </c>
       <c r="AN119" s="1" t="s">
@@ -30423,7 +30423,7 @@
         <v>1206</v>
       </c>
       <c r="BP119" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ119">
         <v>1.58</v>
@@ -30550,7 +30550,7 @@
       <c r="AL120" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM120" s="1" t="s">
+      <c r="AM120" s="22" t="s">
         <v>775</v>
       </c>
       <c r="AN120" s="1" t="s">
@@ -30638,7 +30638,7 @@
         <v>1206</v>
       </c>
       <c r="BP120" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ120">
         <v>1.58</v>
@@ -30765,7 +30765,7 @@
       <c r="AL121" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM121" s="1" t="s">
+      <c r="AM121" s="22" t="s">
         <v>775</v>
       </c>
       <c r="AN121" s="1" t="s">
@@ -30853,7 +30853,7 @@
         <v>1206</v>
       </c>
       <c r="BP121" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ121">
         <v>1.58</v>
@@ -30980,7 +30980,7 @@
       <c r="AL122" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM122" s="1" t="s">
+      <c r="AM122" s="22" t="s">
         <v>775</v>
       </c>
       <c r="AN122" s="1" t="s">
@@ -31068,7 +31068,7 @@
         <v>1206</v>
       </c>
       <c r="BP122" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ122">
         <v>1.58</v>
@@ -31195,7 +31195,7 @@
       <c r="AL123" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM123" s="1" t="s">
+      <c r="AM123" s="22" t="s">
         <v>775</v>
       </c>
       <c r="AN123" s="1" t="s">
@@ -31283,7 +31283,7 @@
         <v>1206</v>
       </c>
       <c r="BP123" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ123">
         <v>1.58</v>
@@ -31410,7 +31410,7 @@
       <c r="AL124" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM124" s="1" t="s">
+      <c r="AM124" s="22" t="s">
         <v>775</v>
       </c>
       <c r="AN124" s="1" t="s">
@@ -31498,7 +31498,7 @@
         <v>1206</v>
       </c>
       <c r="BP124" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ124">
         <v>1.58</v>
@@ -31625,7 +31625,7 @@
       <c r="AL125" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM125" s="1" t="s">
+      <c r="AM125" s="22" t="s">
         <v>775</v>
       </c>
       <c r="AN125" s="1" t="s">
@@ -31713,7 +31713,7 @@
         <v>1206</v>
       </c>
       <c r="BP125" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ125">
         <v>1.58</v>
@@ -31840,7 +31840,7 @@
       <c r="AL126" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM126" s="1" t="s">
+      <c r="AM126" s="22" t="s">
         <v>775</v>
       </c>
       <c r="AN126" s="1" t="s">
@@ -31928,7 +31928,7 @@
         <v>1206</v>
       </c>
       <c r="BP126" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ126">
         <v>1.58</v>
@@ -32055,7 +32055,7 @@
       <c r="AL127" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM127" s="1" t="s">
+      <c r="AM127" s="22" t="s">
         <v>775</v>
       </c>
       <c r="AN127" s="1" t="s">
@@ -32143,7 +32143,7 @@
         <v>1206</v>
       </c>
       <c r="BP127" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ127">
         <v>1.58</v>
@@ -32270,7 +32270,7 @@
       <c r="AL128" s="1" t="s">
         <v>1169</v>
       </c>
-      <c r="AM128" s="1" t="s">
+      <c r="AM128" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN128" s="1" t="s">
@@ -32358,7 +32358,7 @@
         <v>1206</v>
       </c>
       <c r="BP128" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ128" s="1">
         <v>21</v>
@@ -32485,7 +32485,7 @@
       <c r="AL129" s="1" t="s">
         <v>1170</v>
       </c>
-      <c r="AM129" s="1" t="s">
+      <c r="AM129" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN129" s="1" t="s">
@@ -32573,7 +32573,7 @@
         <v>1206</v>
       </c>
       <c r="BP129" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ129" s="1">
         <v>14</v>
@@ -32700,7 +32700,7 @@
       <c r="AL130" s="1" t="s">
         <v>1169</v>
       </c>
-      <c r="AM130" s="1" t="s">
+      <c r="AM130" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN130" s="1" t="s">
@@ -32788,7 +32788,7 @@
         <v>1206</v>
       </c>
       <c r="BP130" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ130" s="1">
         <v>21</v>
@@ -32915,7 +32915,7 @@
       <c r="AL131" s="1" t="s">
         <v>1170</v>
       </c>
-      <c r="AM131" s="1" t="s">
+      <c r="AM131" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN131" s="1" t="s">
@@ -33003,7 +33003,7 @@
         <v>1206</v>
       </c>
       <c r="BP131" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ131" s="1">
         <v>14</v>
@@ -33130,7 +33130,7 @@
       <c r="AL132" s="1" t="s">
         <v>1169</v>
       </c>
-      <c r="AM132" s="1" t="s">
+      <c r="AM132" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN132" s="1" t="s">
@@ -33218,7 +33218,7 @@
         <v>1206</v>
       </c>
       <c r="BP132" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ132" s="1">
         <v>21</v>
@@ -33345,7 +33345,7 @@
       <c r="AL133" s="1" t="s">
         <v>1170</v>
       </c>
-      <c r="AM133" s="1" t="s">
+      <c r="AM133" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN133" s="1" t="s">
@@ -33433,7 +33433,7 @@
         <v>1206</v>
       </c>
       <c r="BP133" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ133" s="1">
         <v>14</v>
@@ -33560,7 +33560,7 @@
       <c r="AL134" s="1" t="s">
         <v>1169</v>
       </c>
-      <c r="AM134" s="1" t="s">
+      <c r="AM134" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN134" s="1" t="s">
@@ -33648,7 +33648,7 @@
         <v>1206</v>
       </c>
       <c r="BP134" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ134" s="1">
         <v>21</v>
@@ -33775,7 +33775,7 @@
       <c r="AL135" s="1" t="s">
         <v>1170</v>
       </c>
-      <c r="AM135" s="1" t="s">
+      <c r="AM135" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN135" s="1" t="s">
@@ -33863,7 +33863,7 @@
         <v>1206</v>
       </c>
       <c r="BP135" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ135" s="1">
         <v>14</v>
@@ -33990,7 +33990,7 @@
       <c r="AL136" s="1" t="s">
         <v>1169</v>
       </c>
-      <c r="AM136" s="1" t="s">
+      <c r="AM136" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN136" s="1" t="s">
@@ -34078,7 +34078,7 @@
         <v>1206</v>
       </c>
       <c r="BP136" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ136" s="1">
         <v>21</v>
@@ -34205,7 +34205,7 @@
       <c r="AL137" s="1" t="s">
         <v>1170</v>
       </c>
-      <c r="AM137" s="1" t="s">
+      <c r="AM137" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN137" s="1" t="s">
@@ -34293,7 +34293,7 @@
         <v>1206</v>
       </c>
       <c r="BP137" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ137" s="1">
         <v>14</v>
@@ -34420,7 +34420,7 @@
       <c r="AL138" s="1" t="s">
         <v>1169</v>
       </c>
-      <c r="AM138" s="1" t="s">
+      <c r="AM138" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN138" s="1" t="s">
@@ -34508,7 +34508,7 @@
         <v>1206</v>
       </c>
       <c r="BP138" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ138" s="1">
         <v>21</v>
@@ -34635,7 +34635,7 @@
       <c r="AL139" s="1" t="s">
         <v>1170</v>
       </c>
-      <c r="AM139" s="1" t="s">
+      <c r="AM139" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN139" s="1" t="s">
@@ -34723,7 +34723,7 @@
         <v>1206</v>
       </c>
       <c r="BP139" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ139" s="1">
         <v>14</v>
@@ -34850,7 +34850,7 @@
       <c r="AL140" s="1" t="s">
         <v>1169</v>
       </c>
-      <c r="AM140" s="1" t="s">
+      <c r="AM140" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN140" s="1" t="s">
@@ -34938,7 +34938,7 @@
         <v>1206</v>
       </c>
       <c r="BP140" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ140" s="1">
         <v>21</v>
@@ -35065,7 +35065,7 @@
       <c r="AL141" s="1" t="s">
         <v>1170</v>
       </c>
-      <c r="AM141" s="1" t="s">
+      <c r="AM141" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN141" s="1" t="s">
@@ -35153,7 +35153,7 @@
         <v>1206</v>
       </c>
       <c r="BP141" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ141" s="1">
         <v>14</v>
@@ -35280,7 +35280,7 @@
       <c r="AL142" s="1" t="s">
         <v>1169</v>
       </c>
-      <c r="AM142" s="1" t="s">
+      <c r="AM142" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN142" s="1" t="s">
@@ -35368,7 +35368,7 @@
         <v>1206</v>
       </c>
       <c r="BP142" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ142" s="1">
         <v>21</v>
@@ -35495,7 +35495,7 @@
       <c r="AL143" s="1" t="s">
         <v>1170</v>
       </c>
-      <c r="AM143" s="1" t="s">
+      <c r="AM143" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN143" s="1" t="s">
@@ -35583,7 +35583,7 @@
         <v>1206</v>
       </c>
       <c r="BP143" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ143" s="1">
         <v>14</v>
@@ -35710,7 +35710,7 @@
       <c r="AL144" s="1" t="s">
         <v>1169</v>
       </c>
-      <c r="AM144" s="1" t="s">
+      <c r="AM144" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN144" s="1" t="s">
@@ -35798,7 +35798,7 @@
         <v>1206</v>
       </c>
       <c r="BP144" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ144" s="1">
         <v>21</v>
@@ -35925,7 +35925,7 @@
       <c r="AL145" s="1" t="s">
         <v>1170</v>
       </c>
-      <c r="AM145" s="1" t="s">
+      <c r="AM145" s="22" t="s">
         <v>650</v>
       </c>
       <c r="AN145" s="1" t="s">
@@ -36013,7 +36013,7 @@
         <v>1206</v>
       </c>
       <c r="BP145" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ145" s="1">
         <v>14</v>
@@ -36140,7 +36140,7 @@
       <c r="AL146" s="1" t="s">
         <v>819</v>
       </c>
-      <c r="AM146" s="1" t="s">
+      <c r="AM146" s="22" t="s">
         <v>775</v>
       </c>
       <c r="AN146" s="1" t="s">
@@ -36228,7 +36228,7 @@
         <v>1206</v>
       </c>
       <c r="BP146" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ146" s="7">
         <v>0.38500000000000001</v>
@@ -36355,7 +36355,7 @@
       <c r="AL147" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM147" s="1" t="s">
+      <c r="AM147" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN147" s="1" t="s">
@@ -36443,7 +36443,7 @@
         <v>1206</v>
       </c>
       <c r="BP147" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ147" s="1">
         <v>10.8</v>
@@ -36570,7 +36570,7 @@
       <c r="AL148" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM148" s="1" t="s">
+      <c r="AM148" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN148" s="1" t="s">
@@ -36658,7 +36658,7 @@
         <v>1206</v>
       </c>
       <c r="BP148" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ148" s="1">
         <v>10.8</v>
@@ -36785,7 +36785,7 @@
       <c r="AL149" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM149" s="1" t="s">
+      <c r="AM149" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN149" s="1" t="s">
@@ -36873,7 +36873,7 @@
         <v>1206</v>
       </c>
       <c r="BP149" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ149" s="1">
         <v>10.8</v>
@@ -37000,7 +37000,7 @@
       <c r="AL150" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM150" s="1" t="s">
+      <c r="AM150" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN150" s="1" t="s">
@@ -37088,7 +37088,7 @@
         <v>1206</v>
       </c>
       <c r="BP150" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ150" s="1">
         <v>10.8</v>
@@ -37215,7 +37215,7 @@
       <c r="AL151" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM151" s="1" t="s">
+      <c r="AM151" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN151" s="1" t="s">
@@ -37303,7 +37303,7 @@
         <v>1206</v>
       </c>
       <c r="BP151" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ151" s="1">
         <v>4.3</v>
@@ -37430,7 +37430,7 @@
       <c r="AL152" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM152" s="1" t="s">
+      <c r="AM152" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN152" s="1" t="s">
@@ -37518,7 +37518,7 @@
         <v>1206</v>
       </c>
       <c r="BP152" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ152" s="1">
         <v>4.3</v>
@@ -37645,7 +37645,7 @@
       <c r="AL153" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM153" s="1" t="s">
+      <c r="AM153" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN153" s="1" t="s">
@@ -37733,7 +37733,7 @@
         <v>1206</v>
       </c>
       <c r="BP153" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ153" s="1">
         <v>1</v>
@@ -37860,7 +37860,7 @@
       <c r="AL154" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM154" s="1" t="s">
+      <c r="AM154" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN154" s="1" t="s">
@@ -37948,7 +37948,7 @@
         <v>1206</v>
       </c>
       <c r="BP154" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ154" s="1">
         <v>1</v>
@@ -38075,7 +38075,7 @@
       <c r="AL155" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM155" s="1" t="s">
+      <c r="AM155" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN155" s="1" t="s">
@@ -38163,7 +38163,7 @@
         <v>1206</v>
       </c>
       <c r="BP155" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ155" s="1">
         <v>1</v>
@@ -38290,7 +38290,7 @@
       <c r="AL156" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM156" s="1" t="s">
+      <c r="AM156" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN156" s="1" t="s">
@@ -38378,7 +38378,7 @@
         <v>1206</v>
       </c>
       <c r="BP156" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ156" s="1">
         <v>1</v>
@@ -38505,7 +38505,7 @@
       <c r="AL157" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM157" s="1" t="s">
+      <c r="AM157" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN157" s="1" t="s">
@@ -38593,7 +38593,7 @@
         <v>1206</v>
       </c>
       <c r="BP157" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ157" s="1">
         <v>1</v>
@@ -38720,7 +38720,7 @@
       <c r="AL158" s="1" t="s">
         <v>919</v>
       </c>
-      <c r="AM158" s="1" t="s">
+      <c r="AM158" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN158" s="1" t="s">
@@ -38808,7 +38808,7 @@
         <v>1206</v>
       </c>
       <c r="BP158" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ158" s="1">
         <v>1</v>
@@ -38935,7 +38935,7 @@
       <c r="AL159" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM159" s="1" t="s">
+      <c r="AM159" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN159" s="1" t="s">
@@ -39150,7 +39150,7 @@
       <c r="AL160" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM160" s="1" t="s">
+      <c r="AM160" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN160" s="1" t="s">
@@ -39365,7 +39365,7 @@
       <c r="AL161" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM161" s="1" t="s">
+      <c r="AM161" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN161" s="1" t="s">
@@ -39453,7 +39453,7 @@
         <v>1206</v>
       </c>
       <c r="BP161" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ161" s="1">
         <v>0.2</v>
@@ -39580,7 +39580,7 @@
       <c r="AL162" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM162" s="1" t="s">
+      <c r="AM162" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN162" s="1" t="s">
@@ -39668,7 +39668,7 @@
         <v>1206</v>
       </c>
       <c r="BP162" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ162" s="1">
         <v>0.2</v>
@@ -39795,7 +39795,7 @@
       <c r="AL163" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM163" s="1" t="s">
+      <c r="AM163" s="22" t="s">
         <v>580</v>
       </c>
       <c r="AN163" s="1" t="s">
@@ -39883,7 +39883,7 @@
         <v>1206</v>
       </c>
       <c r="BP163" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ163" s="1">
         <v>20.486076598151243</v>
@@ -40010,7 +40010,7 @@
       <c r="AL164" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM164" s="1" t="s">
+      <c r="AM164" s="22" t="s">
         <v>580</v>
       </c>
       <c r="AN164" s="1" t="s">
@@ -40098,7 +40098,7 @@
         <v>1206</v>
       </c>
       <c r="BP164" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ164" s="1">
         <v>20.486076598151243</v>
@@ -40225,7 +40225,7 @@
       <c r="AL165" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM165" s="1" t="s">
+      <c r="AM165" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN165" s="1" t="s">
@@ -40313,7 +40313,7 @@
         <v>1206</v>
       </c>
       <c r="BP165" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ165" s="1">
         <v>20.486076598151243</v>
@@ -40440,7 +40440,7 @@
       <c r="AL166" s="1" t="s">
         <v>1134</v>
       </c>
-      <c r="AM166" s="1" t="s">
+      <c r="AM166" s="22" t="s">
         <v>725</v>
       </c>
       <c r="AN166" s="1" t="s">
@@ -40528,7 +40528,7 @@
         <v>1206</v>
       </c>
       <c r="BP166" s="11" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="BQ166" s="1">
         <v>1.37</v>
@@ -40655,7 +40655,7 @@
       <c r="AL167" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM167" s="11" t="s">
+      <c r="AM167" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN167" s="11" t="s">
@@ -40743,7 +40743,7 @@
         <v>1207</v>
       </c>
       <c r="BP167" s="20" t="s">
-        <v>1340</v>
+        <v>1334</v>
       </c>
       <c r="BQ167" s="1">
         <v>0.184668989547038</v>
@@ -40752,7 +40752,7 @@
         <v>30</v>
       </c>
       <c r="BS167" s="1" t="s">
-        <v>1336</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="168" spans="1:71">
@@ -40870,7 +40870,7 @@
       <c r="AL168" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM168" s="11" t="s">
+      <c r="AM168" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN168" s="11" t="s">
@@ -40958,7 +40958,7 @@
         <v>1207</v>
       </c>
       <c r="BP168" s="20" t="s">
-        <v>1340</v>
+        <v>1334</v>
       </c>
       <c r="BQ168" s="1">
         <v>0.184668989547038</v>
@@ -40967,7 +40967,7 @@
         <v>30</v>
       </c>
       <c r="BS168" s="1" t="s">
-        <v>1336</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="169" spans="1:71">
@@ -41085,7 +41085,7 @@
       <c r="AL169" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM169" s="11" t="s">
+      <c r="AM169" s="22" t="s">
         <v>348</v>
       </c>
       <c r="AN169" s="11" t="s">
@@ -41173,7 +41173,7 @@
         <v>1207</v>
       </c>
       <c r="BP169" s="20" t="s">
-        <v>1340</v>
+        <v>1334</v>
       </c>
       <c r="BQ169" s="1">
         <v>0.184668989547038</v>
@@ -41182,7 +41182,7 @@
         <v>30</v>
       </c>
       <c r="BS169" s="1" t="s">
-        <v>1337</v>
+        <v>1331</v>
       </c>
     </row>
     <row r="170" spans="1:71">
@@ -41300,7 +41300,7 @@
       <c r="AL170" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM170" s="11" t="s">
+      <c r="AM170" s="22" t="s">
         <v>348</v>
       </c>
       <c r="AN170" s="11" t="s">
@@ -41388,7 +41388,7 @@
         <v>1207</v>
       </c>
       <c r="BP170" s="20" t="s">
-        <v>1340</v>
+        <v>1334</v>
       </c>
       <c r="BQ170" s="1">
         <v>0.184668989547038</v>
@@ -41397,7 +41397,7 @@
         <v>30</v>
       </c>
       <c r="BS170" s="1" t="s">
-        <v>1337</v>
+        <v>1331</v>
       </c>
     </row>
     <row r="171" spans="1:71">
@@ -41515,7 +41515,7 @@
       <c r="AL171" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM171" s="11" t="s">
+      <c r="AM171" s="22" t="s">
         <v>1122</v>
       </c>
       <c r="AN171" s="11" t="s">
@@ -41730,7 +41730,7 @@
       <c r="AL172" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM172" s="11" t="s">
+      <c r="AM172" s="22" t="s">
         <v>1123</v>
       </c>
       <c r="AO172" s="1">
@@ -41942,7 +41942,7 @@
       <c r="AL173" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM173" s="11" t="s">
+      <c r="AM173" s="22" t="s">
         <v>1126</v>
       </c>
       <c r="AN173" s="11" t="s">
@@ -42157,7 +42157,7 @@
       <c r="AL174" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM174" s="11" t="s">
+      <c r="AM174" s="22" t="s">
         <v>1127</v>
       </c>
       <c r="AN174" s="11" t="s">
@@ -42325,7 +42325,7 @@
         <v>314</v>
       </c>
       <c r="W175" s="1" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="X175" s="11" t="s">
         <v>312</v>
@@ -42372,8 +42372,8 @@
       <c r="AL175" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM175" s="11" t="s">
-        <v>1322</v>
+      <c r="AM175" s="22" t="s">
+        <v>1321</v>
       </c>
       <c r="AN175" s="11" t="s">
         <v>314</v>
@@ -42460,7 +42460,7 @@
         <v>1207</v>
       </c>
       <c r="BP175" s="1" t="s">
-        <v>1342</v>
+        <v>1336</v>
       </c>
       <c r="BQ175" s="1">
         <v>0.2</v>
@@ -42469,7 +42469,7 @@
         <v>26.499666666666666</v>
       </c>
       <c r="BS175" s="1" t="s">
-        <v>1335</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="176" spans="1:71">
@@ -42540,7 +42540,7 @@
         <v>314</v>
       </c>
       <c r="W176" s="1" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="X176" s="11" t="s">
         <v>312</v>
@@ -42587,7 +42587,7 @@
       <c r="AL176" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM176" s="11" t="s">
+      <c r="AM176" s="22" t="s">
         <v>348</v>
       </c>
       <c r="AN176" s="11" t="s">
@@ -42675,7 +42675,7 @@
         <v>1207</v>
       </c>
       <c r="BP176" s="1" t="s">
-        <v>1342</v>
+        <v>1336</v>
       </c>
       <c r="BQ176" s="1">
         <v>0.2</v>
@@ -42684,7 +42684,7 @@
         <v>26.499666666666666</v>
       </c>
       <c r="BS176" s="1" t="s">
-        <v>1334</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="177" spans="1:71">
@@ -42755,7 +42755,7 @@
         <v>314</v>
       </c>
       <c r="W177" s="1" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="X177" s="11" t="s">
         <v>312</v>
@@ -42802,8 +42802,8 @@
       <c r="AL177" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM177" s="11" t="s">
-        <v>1322</v>
+      <c r="AM177" s="22" t="s">
+        <v>1321</v>
       </c>
       <c r="AN177" s="11" t="s">
         <v>314</v>
@@ -42890,7 +42890,7 @@
         <v>1207</v>
       </c>
       <c r="BP177" s="1" t="s">
-        <v>1342</v>
+        <v>1336</v>
       </c>
       <c r="BQ177" s="1">
         <v>0.2</v>
@@ -42899,7 +42899,7 @@
         <v>26.499666666666666</v>
       </c>
       <c r="BS177" s="1" t="s">
-        <v>1334</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="178" spans="1:71">
@@ -42967,7 +42967,7 @@
         <v>1</v>
       </c>
       <c r="V178" s="1" t="s">
-        <v>1327</v>
+        <v>1322</v>
       </c>
       <c r="W178" s="1">
         <v>1981</v>
@@ -43017,7 +43017,7 @@
       <c r="AL178" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM178" s="11" t="s">
+      <c r="AM178" s="22" t="s">
         <v>317</v>
       </c>
       <c r="AN178" s="11" t="s">
@@ -43105,7 +43105,7 @@
         <v>1207</v>
       </c>
       <c r="BP178" s="1" t="s">
-        <v>1342</v>
+        <v>1336</v>
       </c>
       <c r="BQ178" s="1">
         <v>0.2</v>
@@ -43114,7 +43114,7 @@
         <v>26.499666666666666</v>
       </c>
       <c r="BS178" s="1" t="s">
-        <v>1333</v>
+        <v>1327</v>
       </c>
     </row>
     <row r="179" spans="1:71">
@@ -43182,7 +43182,7 @@
         <v>1</v>
       </c>
       <c r="V179" s="1" t="s">
-        <v>1327</v>
+        <v>1322</v>
       </c>
       <c r="W179" s="1">
         <v>1981</v>
@@ -43232,8 +43232,8 @@
       <c r="AL179" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM179" s="11" t="s">
-        <v>1323</v>
+      <c r="AM179" s="22" t="s">
+        <v>317</v>
       </c>
       <c r="AN179" s="11" t="s">
         <v>658</v>
@@ -43320,7 +43320,7 @@
         <v>1207</v>
       </c>
       <c r="BP179" s="1" t="s">
-        <v>1342</v>
+        <v>1336</v>
       </c>
       <c r="BQ179" s="1">
         <v>0.2</v>
@@ -43329,7 +43329,7 @@
         <v>26.499666666666666</v>
       </c>
       <c r="BS179" s="1" t="s">
-        <v>1328</v>
+        <v>1323</v>
       </c>
     </row>
     <row r="180" spans="1:71">
@@ -43397,7 +43397,7 @@
         <v>1</v>
       </c>
       <c r="V180" s="1" t="s">
-        <v>1327</v>
+        <v>1322</v>
       </c>
       <c r="W180" s="1">
         <v>1981</v>
@@ -43447,8 +43447,8 @@
       <c r="AL180" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM180" s="11" t="s">
-        <v>1324</v>
+      <c r="AM180" s="22" t="s">
+        <v>317</v>
       </c>
       <c r="AN180" s="11" t="s">
         <v>658</v>
@@ -43535,7 +43535,7 @@
         <v>1207</v>
       </c>
       <c r="BP180" s="1" t="s">
-        <v>1342</v>
+        <v>1336</v>
       </c>
       <c r="BQ180" s="1">
         <v>0.2</v>
@@ -43544,7 +43544,7 @@
         <v>26.499666666666666</v>
       </c>
       <c r="BS180" s="1" t="s">
-        <v>1329</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="181" spans="1:71">
@@ -43612,7 +43612,7 @@
         <v>1</v>
       </c>
       <c r="V181" s="1" t="s">
-        <v>1327</v>
+        <v>1322</v>
       </c>
       <c r="W181" s="1">
         <v>1981</v>
@@ -43662,8 +43662,8 @@
       <c r="AL181" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM181" s="11" t="s">
-        <v>1325</v>
+      <c r="AM181" s="22" t="s">
+        <v>317</v>
       </c>
       <c r="AN181" s="11" t="s">
         <v>658</v>
@@ -43750,7 +43750,7 @@
         <v>1207</v>
       </c>
       <c r="BP181" s="1" t="s">
-        <v>1342</v>
+        <v>1336</v>
       </c>
       <c r="BQ181" s="1">
         <v>0.2</v>
@@ -43759,7 +43759,7 @@
         <v>26.499666666666666</v>
       </c>
       <c r="BS181" s="1" t="s">
-        <v>1330</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="182" spans="1:71">
@@ -43827,7 +43827,7 @@
         <v>1</v>
       </c>
       <c r="V182" s="1" t="s">
-        <v>1327</v>
+        <v>1322</v>
       </c>
       <c r="W182" s="1">
         <v>1981</v>
@@ -43877,8 +43877,8 @@
       <c r="AL182" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM182" s="11" t="s">
-        <v>348</v>
+      <c r="AM182" s="22" t="s">
+        <v>1344</v>
       </c>
       <c r="AN182" s="11" t="s">
         <v>658</v>
@@ -43965,7 +43965,7 @@
         <v>1207</v>
       </c>
       <c r="BP182" s="1" t="s">
-        <v>1342</v>
+        <v>1336</v>
       </c>
       <c r="BQ182" s="1">
         <v>0.2</v>
@@ -43974,7 +43974,7 @@
         <v>26.499666666666666</v>
       </c>
       <c r="BS182" s="1" t="s">
-        <v>1331</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="183" spans="1:71">
@@ -44042,7 +44042,7 @@
         <v>1</v>
       </c>
       <c r="V183" s="1" t="s">
-        <v>1327</v>
+        <v>1322</v>
       </c>
       <c r="W183" s="1">
         <v>1981</v>
@@ -44092,8 +44092,8 @@
       <c r="AL183" s="11" t="s">
         <v>1134</v>
       </c>
-      <c r="AM183" s="11" t="s">
-        <v>1326</v>
+      <c r="AM183" s="22" t="s">
+        <v>317</v>
       </c>
       <c r="AN183" s="11" t="s">
         <v>658</v>
@@ -44180,7 +44180,7 @@
         <v>1207</v>
       </c>
       <c r="BP183" s="1" t="s">
-        <v>1342</v>
+        <v>1336</v>
       </c>
       <c r="BQ183" s="1">
         <v>0.2</v>
@@ -44189,7 +44189,7 @@
         <v>26.499666666666666</v>
       </c>
       <c r="BS183" s="1" t="s">
-        <v>1332</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="184" spans="1:71">
@@ -44203,7 +44203,6 @@
       <c r="AJ184" s="11"/>
       <c r="AK184" s="11"/>
       <c r="AL184" s="11"/>
-      <c r="AM184" s="11"/>
       <c r="AN184" s="11"/>
     </row>
     <row r="185" spans="1:71">
@@ -44217,14 +44216,12 @@
       <c r="AJ185" s="11"/>
       <c r="AK185" s="11"/>
       <c r="AL185" s="11"/>
-      <c r="AM185" s="11"/>
       <c r="AN185" s="11"/>
     </row>
     <row r="186" spans="1:71">
       <c r="D186" s="1" t="s">
         <v>566</v>
       </c>
-      <c r="AM186" s="11"/>
     </row>
     <row r="187" spans="1:71">
       <c r="D187" s="1" t="s">

</xml_diff>

<commit_message>
specifying proxy for Cognie paper
</commit_message>
<xml_diff>
--- a/Output/Data/meta_analysis_data.xlsx
+++ b/Output/Data/meta_analysis_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emlim/Documents/PhD/Ch1-Meta-analysis/Output/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F30B687-9AC0-7A4C-B017-554736D137CF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F93A5E7A-7308-9948-94BD-693409FCCD58}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1220" yWindow="460" windowWidth="26780" windowHeight="15940" activeTab="2" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
+    <workbookView xWindow="1220" yWindow="460" windowWidth="26780" windowHeight="15940" xr2:uid="{40EEFA15-B542-CE42-935C-BBE1E5D9457F}"/>
   </bookViews>
   <sheets>
     <sheet name="Include" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13622" uniqueCount="1426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13640" uniqueCount="1426">
   <si>
     <t>paper_num</t>
   </si>
@@ -37959,6 +37959,9 @@
       <c r="BT136" s="11" t="s">
         <v>1258</v>
       </c>
+      <c r="BU136" s="11" t="s">
+        <v>1259</v>
+      </c>
       <c r="BV136" s="11" t="s">
         <v>314</v>
       </c>
@@ -38199,6 +38202,9 @@
       <c r="BT137" s="11" t="s">
         <v>1258</v>
       </c>
+      <c r="BU137" s="11" t="s">
+        <v>1259</v>
+      </c>
       <c r="BV137" s="11" t="s">
         <v>314</v>
       </c>
@@ -38439,6 +38445,9 @@
       <c r="BT138" s="11" t="s">
         <v>1258</v>
       </c>
+      <c r="BU138" s="11" t="s">
+        <v>1259</v>
+      </c>
       <c r="BV138" s="11" t="s">
         <v>314</v>
       </c>
@@ -38679,6 +38688,9 @@
       <c r="BT139" s="11" t="s">
         <v>1258</v>
       </c>
+      <c r="BU139" s="11" t="s">
+        <v>1259</v>
+      </c>
       <c r="BV139" s="11" t="s">
         <v>314</v>
       </c>
@@ -38919,6 +38931,9 @@
       <c r="BT140" s="11" t="s">
         <v>1258</v>
       </c>
+      <c r="BU140" s="11" t="s">
+        <v>1259</v>
+      </c>
       <c r="BV140" s="11" t="s">
         <v>314</v>
       </c>
@@ -39159,6 +39174,9 @@
       <c r="BT141" s="11" t="s">
         <v>1258</v>
       </c>
+      <c r="BU141" s="11" t="s">
+        <v>1259</v>
+      </c>
       <c r="BV141" s="11" t="s">
         <v>314</v>
       </c>
@@ -39399,6 +39417,9 @@
       <c r="BT142" s="11" t="s">
         <v>1258</v>
       </c>
+      <c r="BU142" s="11" t="s">
+        <v>1259</v>
+      </c>
       <c r="BV142" s="11" t="s">
         <v>314</v>
       </c>
@@ -39639,6 +39660,9 @@
       <c r="BT143" s="11" t="s">
         <v>1258</v>
       </c>
+      <c r="BU143" s="11" t="s">
+        <v>1259</v>
+      </c>
       <c r="BV143" s="11" t="s">
         <v>314</v>
       </c>
@@ -39879,6 +39903,9 @@
       <c r="BT144" s="11" t="s">
         <v>1258</v>
       </c>
+      <c r="BU144" s="11" t="s">
+        <v>1259</v>
+      </c>
       <c r="BV144" s="11" t="s">
         <v>314</v>
       </c>
@@ -40119,6 +40146,9 @@
       <c r="BT145" s="11" t="s">
         <v>1258</v>
       </c>
+      <c r="BU145" s="11" t="s">
+        <v>1259</v>
+      </c>
       <c r="BV145" s="11" t="s">
         <v>314</v>
       </c>
@@ -40359,6 +40389,9 @@
       <c r="BT146" s="11" t="s">
         <v>1258</v>
       </c>
+      <c r="BU146" s="11" t="s">
+        <v>1259</v>
+      </c>
       <c r="BV146" s="11" t="s">
         <v>314</v>
       </c>
@@ -40599,6 +40632,9 @@
       <c r="BT147" s="11" t="s">
         <v>1258</v>
       </c>
+      <c r="BU147" s="11" t="s">
+        <v>1259</v>
+      </c>
       <c r="BV147" s="11" t="s">
         <v>314</v>
       </c>
@@ -40839,6 +40875,9 @@
       <c r="BT148" s="11" t="s">
         <v>1258</v>
       </c>
+      <c r="BU148" s="11" t="s">
+        <v>1259</v>
+      </c>
       <c r="BV148" s="11" t="s">
         <v>314</v>
       </c>
@@ -41079,6 +41118,9 @@
       <c r="BT149" s="11" t="s">
         <v>1258</v>
       </c>
+      <c r="BU149" s="11" t="s">
+        <v>1259</v>
+      </c>
       <c r="BV149" s="11" t="s">
         <v>314</v>
       </c>
@@ -41319,6 +41361,9 @@
       <c r="BT150" s="11" t="s">
         <v>1258</v>
       </c>
+      <c r="BU150" s="11" t="s">
+        <v>1259</v>
+      </c>
       <c r="BV150" s="11" t="s">
         <v>314</v>
       </c>
@@ -41559,6 +41604,9 @@
       <c r="BT151" s="11" t="s">
         <v>1258</v>
       </c>
+      <c r="BU151" s="11" t="s">
+        <v>1259</v>
+      </c>
       <c r="BV151" s="11" t="s">
         <v>314</v>
       </c>
@@ -41799,6 +41847,9 @@
       <c r="BT152" s="11" t="s">
         <v>1258</v>
       </c>
+      <c r="BU152" s="11" t="s">
+        <v>1259</v>
+      </c>
       <c r="BV152" s="11" t="s">
         <v>314</v>
       </c>
@@ -42038,6 +42089,9 @@
       </c>
       <c r="BT153" s="11" t="s">
         <v>1258</v>
+      </c>
+      <c r="BU153" s="11" t="s">
+        <v>1259</v>
       </c>
       <c r="BV153" s="11" t="s">
         <v>314</v>

</xml_diff>